<commit_message>
Update the event catalog row for Event 34 Industrial Boom
Event 34 carries the Event Details wording and the three evolution descriptions that match the in-game text, Positive Economy cluster 7 and the Needs Testing status. The generated CSV exports are refreshed from the workbook. The same workbook save also holds the concurrent Event 37 row text.
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -3636,7 +3636,7 @@
       <c r="K30" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="L30" s="54"/>
+      <c r="L30" s="54" t="n"/>
       <c r="M30" s="72" t="inlineStr">
         <is>
           <t>Needs Testing</t>
@@ -3868,12 +3868,24 @@
       </c>
       <c r="C35" s="30" t="inlineStr">
         <is>
-          <t>The expansion records its overheating, reserves, projects, supplier ties, regions, and reach. A hard landing turns those strengths and liabilities into the opening conditions of Great Depression 2.0.</t>
-        </is>
-      </c>
-      <c r="D35" s="35" t="n"/>
-      <c r="E35" s="36" t="n"/>
-      <c r="F35" s="37" t="n"/>
+          <t>A major power or a player government experiences an industrial acceleration far beyond what its factories, railways and workers should allow. The extra output arrives at once. Keeping it from breaking the economy is the hard part, and a boom that is pushed too far ends in a depression.</t>
+        </is>
+      </c>
+      <c r="D35" s="35" t="inlineStr">
+        <is>
+          <t>Credit and confidence carry the boom past what the factories can deliver. Firms announce works before the materials exist, speculative projects are offered to the government, and restraining the banks costs stability.</t>
+        </is>
+      </c>
+      <c r="E35" s="36" t="inlineStr">
+        <is>
+          <t>Chosen regions develop faster than their materials allow. Halls and railways are finished ahead of every schedule, and the works that grow this way leave greater gains behind, if they survive the pressure.</t>
+        </is>
+      </c>
+      <c r="F35" s="37" t="inlineStr">
+        <is>
+          <t>Industry spreads from its centres into neighbouring districts faster than any administration can follow. The government can direct the spread, let it run or contain it, and a collapse now drags the whole world economy down.</t>
+        </is>
+      </c>
       <c r="G35" s="38" t="n"/>
       <c r="H35" s="39" t="n"/>
       <c r="I35" s="40" t="n"/>
@@ -3892,7 +3904,7 @@
       </c>
       <c r="M35" s="72" t="inlineStr">
         <is>
-          <t>To Be Reworked</t>
+          <t>Needs Testing</t>
         </is>
       </c>
     </row>
@@ -3997,12 +4009,24 @@
       </c>
       <c r="C38" s="30" t="inlineStr">
         <is>
-          <t>A major country receives millions of unexplained new recruits.</t>
-        </is>
-      </c>
-      <c r="D38" s="35" t="n"/>
-      <c r="E38" s="36" t="n"/>
-      <c r="F38" s="37" t="n"/>
+          <t>People with homes, families and histories appear overnight in every inhabited land, and their neighbours cannot remember a time without them. The arrivals repeat, and each wave needs houses, work and food before the next one comes. Nobody knows where they come from.</t>
+        </is>
+      </c>
+      <c r="D38" s="35" t="inlineStr">
+        <is>
+          <t>Each manifestation brings far more people, enough to fill new streets in every town.</t>
+        </is>
+      </c>
+      <c r="E38" s="36" t="inlineStr">
+        <is>
+          <t>Manifestations outgrow the housing and food of crowded regions.</t>
+        </is>
+      </c>
+      <c r="F38" s="37" t="inlineStr">
+        <is>
+          <t>Manifestations grow large enough to swamp whole countries, and governments begin counting origins.</t>
+        </is>
+      </c>
       <c r="G38" s="38" t="n"/>
       <c r="H38" s="39" t="n"/>
       <c r="I38" s="40" t="n"/>
@@ -4019,9 +4043,9 @@
           <t>15</t>
         </is>
       </c>
-      <c r="M38" s="72" t="inlineStr">
-        <is>
-          <t>To Be Reworked</t>
+      <c r="M38" s="70" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
         </is>
       </c>
     </row>
@@ -22979,10 +23003,10 @@
       <c r="C37" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="54"/>
-      <c r="G37" s="5"/>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="54" t="n"/>
+      <c r="G37" s="5" t="n"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="4" t="n">
@@ -23625,10 +23649,10 @@
       <c r="C61" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D61" s="5"/>
-      <c r="E61" s="5"/>
-      <c r="F61" s="54"/>
-      <c r="G61" s="5"/>
+      <c r="D61" s="5" t="n"/>
+      <c r="E61" s="5" t="n"/>
+      <c r="F61" s="54" t="n"/>
+      <c r="G61" s="5" t="n"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="4" t="n"/>
@@ -24326,7 +24350,7 @@
       </c>
       <c r="C8" s="52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sovereign Scatter: Every viable independence movement breaks away. Hosts keep a protected remnant, each new state gets its own starting territory, and none joins a league or faction. Intensity changes territory, forces, and pressure.
+          <t>Sovereign Scatter: Every viable independence movement breaks away. Hosts keep a protected remnant, each new state gets its own starting territory, and none joins a league or faction. Intensity changes territory, forces, and pressure.
 Open Congress: Every viable independence movement breaks away from a protected host. The new states join an informal congress, and higher intensity strengthens its charter and shared reserve.
 Separation Wars: Every viable independence movement breaks away. A new state able to confront its former host may open one war of separation. The others receive a regional threat mission.
 Host Wars: Every viable independence movement breaks away. Each new state may open one war against its former host. Hosts keep their homelands, and wars that cannot start become regional threat missions.
@@ -24338,12 +24362,12 @@
       </c>
       <c r="D8" s="52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sovereign Scatter, Open Congress, Separation Wars, Host Wars, Neighbor Wars, Outsider Wars, Patron Worlds, Great Partition</t>
+          <t>Sovereign Scatter, Open Congress, Separation Wars, Host Wars, Neighbor Wars, Outsider Wars, Patron Worlds, Great Partition</t>
         </is>
       </c>
       <c r="E8" s="52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low: Each release gets only its starting territory, fragile defenses, scarce stocks, weak institutions, low recognition, and severe instability.
+          <t>Low: Each release gets only its starting territory, fragile defenses, scarce stocks, weak institutions, low recognition, and severe instability.
 Medium: Releases receive compact territory, militia and border formations, baseline institutions, and ordinary route access.
 High: Releases receive wider territory where borders allow, armed forces, stronger depots and officers, firmer institutions, and faster ambitions.
 Maximum: Releases receive the largest territory and forces, rare support where their route allows it, high-chaos access, early formable discovery, and aggressive AI.</t>

</xml_diff>

<commit_message>
Finish Event 025 for release: seizure restitution, Forerunner Craft test and catalog row
Seized material now returns exactly: the victim keeps one targeted claim per
fragment slot plus the crews actually detained, and an accepted demand returns
them through the physical ledger. A matched, unanswered demand is consumed
before anything moves, so repeated or misdirected answers do nothing. Turning
the survivor's trace at a rival shares the rival-agent cooldown with jamming
and the rival operations, and moved-fragment incidents cannot lose more survey
evidence than the expedition holds. Casualty lines now appear in the three
field-loss reports.

The report picture test reads the shared picture sprites that the Forerunner
Craft uses after its move from slot 36. The event catalog row carries the
Event Details and the five evolution descriptions and is set to Needs Testing.
The completion, limitation and arbitration documents describe the current state.
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -3435,14 +3435,34 @@
       </c>
       <c r="C26" s="30" t="inlineStr">
         <is>
-          <t>A race for alien technology in Antarctica can unlock advanced jet research for the country that secures the site.</t>
-        </is>
-      </c>
-      <c r="D26" s="35" t="n"/>
-      <c r="E26" s="36" t="n"/>
-      <c r="F26" s="37" t="n"/>
-      <c r="G26" s="38" t="n"/>
-      <c r="H26" s="39" t="n"/>
+          <t>Impossible readings beneath the Antarctic ice draw governments into a race across six field sectors. Each expedition keeps a private record of its route, camp, survey evidence and fragments, while five independent hazards can change the race. One expedition secures the primary alien-derived result; every other expedition keeps only what it verified.\n\n§YThe race has not begun in this campaign.§!</t>
+        </is>
+      </c>
+      <c r="D26" s="35" t="inlineStr">
+        <is>
+          <t>The buried transmitter answers field instruments in a patient, non-human pattern, and it grows louder week by week. Strong pulses can burn out radios, drain a camp, injure field crews, scramble survey records or show rivals where an expedition works; shielded instruments and distant listening posts blunt them. The signal adds danger to the race without removing the possibility of recovery.</t>
+        </is>
+      </c>
+      <c r="E26" s="36" t="inlineStr">
+        <is>
+          <t>Movement has been observed beyond the wreck's outer shell. It may be a mechanism, a biological response, or an echo in the snow. Camps report strange tracks, opened compartments, cut cables, moved fragments, missing men and voices on the radio. Each expedition chooses whether to avoid it, guard against it, offer it a path, turn it toward a rival or try to capture it, while the recovery race continues.</t>
+        </is>
+      </c>
+      <c r="F26" s="37" t="inlineStr">
+        <is>
+          <t>Armed patrols and emergency claims are joining the expedition flags. Escorts, blockades, seizures and interceptions push the ice from guarded toward open clash, and every camp grows more exposed as it does. A poorly defended camp can be stormed and stripped of its records and fragments. Rescues and demilitarised corridors, which a rival must accept, pull the crisis back without forcing a global war.</t>
+        </is>
+      </c>
+      <c r="G26" s="38" t="inlineStr">
+        <is>
+          <t>The alien-derived wreck is shedding hot fragments into six distinct sectors. Its integrity falls with time, pulses, fighting near the site, cutting and failed extractions, and only rare stabilisation slows it. Below half integrity unrecovered fields are buried or destroyed, and pieces cut from a failing hull can come out contaminated. If the hull breaks, the command core remains the race's prize.</t>
+        </is>
+      </c>
+      <c r="H26" s="39" t="inlineStr">
+        <is>
+          <t>The recovered system is beginning to anticipate its operators. Dependence remains measurable and recoverable, but each custody decision changes the relationship between human judgment and the alien-derived interface.</t>
+        </is>
+      </c>
       <c r="I26" s="40" t="n"/>
       <c r="J26" s="66" t="inlineStr">
         <is>
@@ -3453,9 +3473,9 @@
         <v>1</v>
       </c>
       <c r="L26" s="54" t="n"/>
-      <c r="M26" s="72" t="inlineStr">
-        <is>
-          <t>To Be Reworked</t>
+      <c r="M26" s="70" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finish Event 32 for release: programme-wide survey, US text, shared fixes
The launch-state survey freezes the full eligible pool and the best-scoring state before payment and no longer needs a map target. Primary-site selection prefers an upgradeable site, rejects wasteland and defers an empty result. The region lookup and the civil-war split bind their actual country instead of the event ROOT. Player text, achievements and the catalog row use US spelling and drop implementation wording from the failed-setup event. The unused missiles_cost constant table is removed, the stale scope and transaction tests follow the new survey contract, and Event 27 moves to Needs Testing in the catalog.
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -3569,7 +3569,7 @@
       </c>
       <c r="M28" s="72" t="inlineStr">
         <is>
-          <t>To Be Reworked</t>
+          <t>Needs Testing</t>
         </is>
       </c>
     </row>
@@ -3782,12 +3782,12 @@
       </c>
       <c r="C33" s="30" t="inlineStr">
         <is>
-          <t>Missile programmes have spread across the world. Countries can build and harden launch sites, stock operational missiles, improve guidance, and secure the officers and codes that control them. Heavier arsenals, guidance failures, special warheads, rogue commands, and automatic retaliation can transform the crisis.</t>
+          <t>Missile programs have spread across the world. Countries can build and harden launch sites, stock operational missiles, improve guidance, and secure the officers and codes that control them. Heavier arsenals, guidance failures, special warheads, rogue commands, and automatic retaliation can transform the crisis.</t>
         </is>
       </c>
       <c r="D33" s="35" t="inlineStr">
         <is>
-          <t>Countries with working launch sites and enough industry can adopt a saturation doctrine for massed salvos. Saturation attacks can overwhelm defences, but they consume many missiles and strain readiness and command control.</t>
+          <t>Countries with working launch sites and enough industry can adopt a saturation doctrine for massed salvos. Saturation attacks can overwhelm defenses, but they consume many missiles and strain readiness and command control.</t>
         </is>
       </c>
       <c r="E33" s="36" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="F33" s="37" t="inlineStr">
         <is>
-          <t>Countries that already possess chemical, biological, nuclear, or thermonuclear weapons can adapt them for missile delivery. Each launch still requires an authorised warhead held in secure custody.</t>
+          <t>Countries that already possess chemical, biological, nuclear, or thermonuclear weapons can adapt them for missile delivery. Each launch still requires an authorized warhead held in secure custody.</t>
         </is>
       </c>
       <c r="G33" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Align the catalog Details for Events 1, 3 and 4 with the in-game Event Details
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -2078,8 +2078,8 @@
       </c>
       <c r="C2" s="30" t="inlineStr">
         <is>
-          <t>Communist organizers turn propaganda networks and local agitation into control of vulnerable states. As their foothold deepens, agitation can harden into insurgent strongholds and lockdowns, raising the risk of revolt.
-Governments can intervene locally or launch a broader emergency response. Delay gives the movement more chances to spread, stage unexpected uprisings, and draw the country toward revolution.</t>
+          <t>Communist organizers turn propaganda networks and local agitation into control of vulnerable states. Strikes give way to committees, committees begin to give orders of their own, and the longer a government waits the closer its country comes to open revolution.
+Governments can answer with local crackdowns or a national emergency operation, and either can go wrong.</t>
         </is>
       </c>
       <c r="D2" s="82" t="inlineStr">
@@ -2194,7 +2194,9 @@
       </c>
       <c r="C4" s="30" t="inlineStr">
         <is>
-          <t>A Himalayan refuge can become the Holy Realm as its people develop a Bodhisattva-led order, the Arhat Administration, and the Buddha Mandate. Political and spiritual choices shape whether the state follows restraint, peacekeeping, coercive pacification, Divine Sovereignty, or the final doctrine.</t>
+          <t>The Holy Realm begins in the Himalayan passes, where a Bodhisattva leads monks and refugees toward a guarded refuge. Its vows shape how the Arhats govern and how envoys approach distant courts.
+As suffering spreads, the Realm's promise of mercy hardens into military doctrine. The Mandala reaches beyond the mountains, and its members must decide whether their vows can survive the pressure of the world around them.
+Final Silence can end in two ways. If Chaos exceeds 1000 and no other ending has begun, the last order calls Fallout upon the world. Otherwise the Empty Seat follows and the world continues.</t>
         </is>
       </c>
       <c r="D4" s="82" t="inlineStr">
@@ -2253,7 +2255,8 @@
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>Wars erupt between eligible countries and expand into linked conflict webs as chaos rises. Special countries can join later stages, turning a local declaration into a wider chain of fighting.</t>
+          <t>Random War turns border orders, panicked ultimatums and opportunistic claims into sudden declarations between sovereign countries.
+As the world grows more unstable, a single incident can pull in neighbors, great powers and stranger states, until a quarrel between two countries has become a chain of wars.</t>
         </is>
       </c>
       <c r="D5" s="82" t="inlineStr">

</xml_diff>

<commit_message>
Align the catalog Event Details and evolution text for Events 10, 11 and 15 with the game
Event 10 now carries the in-game Event Details, the five evolution stages and the Last Shores branch. Event 11 mirrors the opening Event Details. Event 15 mirrors the Event Details and the two later evolution descriptions.
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -2610,40 +2610,37 @@
       </c>
       <c r="C11" s="30" t="inlineStr">
         <is>
-          <t>Death begins in silence on a remote island. Ships stop returning, settlements empty, and the Black Ledger reaches toward other islands before turning to the mainland.
-Every state Death consumes is emptied of its people and reduced to a wasteland. The dead feed Death's soul power, which it spends to spread, raise ghost hosts, and open new footholds. Retaking land does not restore it, and survivors must invest in making the dead zones usable again.
-Living countries can investigate the disappearances, guard their coasts, build quarantine lines, join the Living Compact, and prepare troops for the wastelands. Death is defeated only when every state under its control has been reclaimed.</t>
+          <t>The islands fall silent, and governments search the coast for an answer. A cold presence gathers beyond the sea, where ships, letters, and radio calls no longer return.</t>
         </is>
       </c>
       <c r="D11" s="82" t="inlineStr">
         <is>
-          <t>Death reaches a second island and empties it slowly enough to resemble lost shipping or an abandoned harbor. The silence spreads from shore to shore while mainland governments remain uncertain of its cause.</t>
+          <t>Ships stop arriving from a second island. Nobody yet knows it is lost, but its neighbors have noticed the silence.</t>
         </is>
       </c>
       <c r="E11" s="83" t="inlineStr">
         <is>
-          <t>The Black Ledger reaches the mainland. Coastal settlements empty, survivors name the force consuming them, and the first organized war against Death begins.</t>
+          <t>Death reaches the mainland coast. Coastal settlements fall silent, survivors name the force, and the first armies meet it.</t>
         </is>
       </c>
       <c r="F11" s="84" t="inlineStr">
         <is>
-          <t>Weak ghost hosts rise from emptied land and gather along its borders. They defend the wasteland in broken ranks while Death prepares a larger army from those it has counted.</t>
+          <t>Weak ghost hosts stand in broken ranks around the emptied land. Their shadows mark the first boundary between living towns and the dead.</t>
         </is>
       </c>
       <c r="G11" s="85" t="inlineStr">
         <is>
-          <t>The hollow hosts return in greater numbers and hold their ranks longer. They remain imperfect soldiers, yet every fallen district gives Death more ground from which to raise them.</t>
+          <t>Hollow hosts gather in greater numbers and hold the front. More towns fall silent, while the living find fewer routes out.</t>
         </is>
       </c>
       <c r="H11" s="86" t="inlineStr">
         <is>
-          <t>An emptied continent becomes Death's muster ground. Ghost hosts cross the last shores in force and attack the living wherever the Black Ledger remains unfinished.</t>
+          <t>A continent falls silent, and Death's forces turn toward the last occupied shores. Few governments still have room to retreat.</t>
         </is>
       </c>
       <c r="I11" s="87" t="inlineStr">
         <is>
-          <t>Death has emptied enough land to turn islands, wastelands, and ghost hosts into one design. A consumed continent gives Zol the ground from which to reach every surviving shore.
-New footholds open across the living world, and the dead march from the last shores to complete the Black Ledger. No population remains beyond Death's count.</t>
+          <t>Death has begun its Last Shores campaign. The living countries that remain must hold distant fronts across empty cities and ruined supply roads.</t>
         </is>
       </c>
       <c r="J11" s="65" t="inlineStr">
@@ -2672,7 +2669,7 @@
       </c>
       <c r="C12" s="30" t="inlineStr">
         <is>
-          <t>A covert alliance leaves the same traces in distant incidents. Couriers vanish, equipment fails, and quiet methods recur across borders. Following the pattern can expose the network before its next operation.</t>
+          <t>Strangers keep meeting in the wrong places. Couriers vanish, equipment fails, and the same quiet methods turn up in distant incidents. Nobody can say who is behind them.</t>
         </is>
       </c>
       <c r="D12" s="82" t="inlineStr">
@@ -2898,7 +2895,7 @@
       </c>
       <c r="C16" s="30" t="inlineStr">
         <is>
-          <t>A translated manifesto slips out of reading rooms and into the government of a small country. It promises that common stores, useful work, and public need can build a fairer society. Its readers divide over who decides what people need and how much freedom the plan can afford. Shortages, public works, local charters, and deals with neighbors put every promise to the test.</t>
+          <t>A translated manifesto slips out of reading rooms and into the government of a small country. It promises that common stores, useful work, and public need can build a fairer society. Its readers quickly split over who gets to decide what people need and how much freedom the plan can afford.\n\nShortages, public works, local charters, and deals with neighboring states put every promise to the test. The commonwealth must prove that it can care for people without turning necessity into an excuse for control or conquest.</t>
         </is>
       </c>
       <c r="D16" s="82" t="inlineStr">
@@ -2918,12 +2915,12 @@
       </c>
       <c r="G16" s="85" t="inlineStr">
         <is>
-          <t>The manifesto now has a place in regional politics. Governments quote it when they ask for aid, defend local charters, refuse threats, or seek association. Small states must decide whether the commonwealth looks like a refuge, a useful partner, or an ambitious neighbor.</t>
+          <t>The manifesto now shapes regional politics. Governments invoke it to seek aid, defend local charters, resist threats, or ask for association, and small states must decide whether the commonwealth is a refuge, a useful partner, or an ambitious neighbor.</t>
         </is>
       </c>
       <c r="H16" s="86" t="inlineStr">
         <is>
-          <t>The world around the commonwealth is coming apart. Reserve trains, guarded harbors, refugee districts, fortifications, and member councils all compete for the same supplies. One path closes the gates and demands service from everyone inside. The other shares refuge among willing towns and spreads the burden across the league.</t>
+          <t>The world around the commonwealth is coming apart. Harbors, trains, fortifications, and refuge towns all need the same stores. Citizens and League members ask whether the gates will protect them, who must serve inside, and which neighbors will share the burden.</t>
         </is>
       </c>
       <c r="I16" s="40" t="n"/>

</xml_diff>

<commit_message>
Align the Event 17, 19 and 20 catalog details with the in-game Event Details text
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -3012,7 +3012,8 @@
       </c>
       <c r="C18" s="30" t="inlineStr">
         <is>
-          <t>A small neutral country is running out of room to stand alone. The great blocs offer protection, weapons, and a seat at their table, sending their envoys toward the next exposed border. Neutrality becomes a political and military struggle fought through councils, troops, and public resolve.</t>
+          <t>A small neutral country is running out of room to stand alone. The great blocs offer protection, weapons, and a seat at their table. Refusing every bloc can leave the country exposed.
+The winning faction will worry nearby neutrals and send its envoys toward the next exposed border. Neutrality becomes something a country must defend with speeches, councils, troops, and a fair bit of nerve.</t>
         </is>
       </c>
       <c r="D18" s="82" t="inlineStr">
@@ -3123,13 +3124,13 @@
       </c>
       <c r="C20" s="30" t="inlineStr">
         <is>
-          <t>Fully formed military units are appearing across the world with no recruitment orders, training records, or known home. Governments suddenly have to feed, equip, command, and watch soldiers who arrived ready to march.
+          <t>Fully formed military units are appearing across the world with no recruitment orders, training history, or known home. Governments suddenly have to feed, equip, command, and watch soldiers who arrived ready to march.
 Some formations bring strange weapons, ambitious commanders, or troops that are not human at all. A useful windfall can become a rival army very quickly.</t>
         </is>
       </c>
       <c r="D20" s="82" t="inlineStr">
         <is>
-          <t>The soldiers from nowhere now have district staffs, proper rolls, and officers the government can actually hold responsible.</t>
+          <t>The soldiers from nowhere have district staffs, proper rolls, and officers the government can actually hold responsible.</t>
         </is>
       </c>
       <c r="E20" s="83" t="inlineStr">
@@ -3180,7 +3181,7 @@
       <c r="C21" s="30" t="inlineStr">
         <is>
           <t>A black-marked fever has broken out on the mainland. It moves through roads, ports, hungry cities, and rat-filled ruins, leaving governments to choose which places to isolate and which people they can still save.
-If the plague is allowed to settle in, the rats may become something more dangerous than carriers. Whole warrens can learn to fight, govern, and follow a king of their own.</t>
+If the plague is allowed to settle in, the rats may become something more dangerous than carriers.</t>
         </is>
       </c>
       <c r="D21" s="82" t="inlineStr">

</xml_diff>

<commit_message>
Mirror the renamed event names for Events 23, 54, 58, 61, 65, 66, 74, 82, 93 and 96 in the event catalog
Events sheet names and the matching Cluster Memberships display names now equal the localised event names; CSV exports regenerated.
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -3333,7 +3333,7 @@
       </c>
       <c r="B24" s="30" t="inlineStr">
         <is>
-          <t>SOV Nuclear Bombs</t>
+          <t>Soviet Nuclear Bombs</t>
         </is>
       </c>
       <c r="C24" s="30" t="inlineStr">
@@ -4735,7 +4735,7 @@
       </c>
       <c r="B55" s="30" t="inlineStr">
         <is>
-          <t>Gift from scientists</t>
+          <t>New Technology</t>
         </is>
       </c>
       <c r="C55" s="30" t="inlineStr">
@@ -4891,7 +4891,7 @@
       </c>
       <c r="B59" s="30" t="inlineStr">
         <is>
-          <t>The Industrial Complex</t>
+          <t>Industrial Complexes</t>
         </is>
       </c>
       <c r="C59" s="30" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="B62" s="30" t="inlineStr">
         <is>
-          <t>Half mils into civs</t>
+          <t>Arms Factory Conversion</t>
         </is>
       </c>
       <c r="C62" s="30" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="B66" s="30" t="inlineStr">
         <is>
-          <t>Random Trait</t>
+          <t>Random Leader Trait</t>
         </is>
       </c>
       <c r="C66" s="30" t="inlineStr">
@@ -5199,7 +5199,7 @@
       </c>
       <c r="B67" s="30" t="inlineStr">
         <is>
-          <t>CIC</t>
+          <t>Construction Industrial Capacity</t>
         </is>
       </c>
       <c r="C67" s="30" t="inlineStr">
@@ -5465,7 +5465,7 @@
       </c>
       <c r="B75" s="30" t="inlineStr">
         <is>
-          <t>Japan lands in USA</t>
+          <t>Japan in California</t>
         </is>
       </c>
       <c r="C75" s="30" t="inlineStr">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="B83" s="30" t="inlineStr">
         <is>
-          <t>Law upgrade</t>
+          <t>Step Toward Mobilization</t>
         </is>
       </c>
       <c r="C83" s="30" t="inlineStr">
@@ -6134,7 +6134,7 @@
       </c>
       <c r="B94" s="30" t="inlineStr">
         <is>
-          <t>Portugal wants land</t>
+          <t>Portugal Demands Galicia</t>
         </is>
       </c>
       <c r="C94" s="30" t="inlineStr">
@@ -6239,7 +6239,7 @@
       </c>
       <c r="B97" s="30" t="inlineStr">
         <is>
-          <t>Divisions lock</t>
+          <t>Division Templates Locked</t>
         </is>
       </c>
       <c r="C97" s="30" t="inlineStr">
@@ -22654,7 +22654,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Return to Peacetime</t>
+          <t>Arms Factory Conversion</t>
         </is>
       </c>
       <c r="F24" s="54" t="inlineStr">
@@ -23139,7 +23139,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Random Buildings</t>
+          <t>Industrial Complexes</t>
         </is>
       </c>
       <c r="F41" s="54" t="inlineStr">
@@ -23251,7 +23251,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Random Tech</t>
+          <t>New Technology</t>
         </is>
       </c>
       <c r="F45" s="54" t="inlineStr">
@@ -23278,7 +23278,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Random Trait</t>
+          <t>Random Leader Trait</t>
         </is>
       </c>
       <c r="F46" s="54" t="inlineStr">

</xml_diff>

<commit_message>
Align the Event 21, 23 and 26 catalog rows with the in-game text
Event 21 Details, Evo I and Evo II follow the current Event Details and evolution wording, Event 23 moves to Needs Testing, and Event 26 Details and Evo I follow the current premise and the rest-of-the-day wording.
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -3244,7 +3244,7 @@
       </c>
       <c r="C22" s="30" t="inlineStr">
         <is>
-          <t>A country's chain of command has split between rival political and military authorities. Capitals, supply routes, public legitimacy, and the terms offered to each front will shape the conflict.
+          <t>A country's chain of command has split between rival political and military authorities. Capitals, supply routes, public legitimacy, and the terms offered to each front will shape the conflict. When the fronts gather, a war already under way can draw in new regional sides, or its government and claimants take firmer command of the fronts they hold. A claimant that replaces the government can open a new war against the old government's foreign enemies for its own core or claimed territory, or let that quarrel lapse.
 Settlement
 The sides have accepted terms based on recognition, autonomy, coalition, partition, or disarmament. The peace will last only if every signatory meets its obligations.
 Reconstruction
@@ -3253,12 +3253,12 @@
       </c>
       <c r="D22" s="35" t="inlineStr">
         <is>
-          <t>Additional commands and regional movements have entered the first war. Several rival authorities are now competing for capitals, supply routes, and terms of peace.</t>
+          <t>Rival commands and regional movements are joining the civil wars already under way. Where a region can hold its own capital and forces, a new side takes up arms; elsewhere, governments and claimants tighten their grip on their fronts. New crises can now open on several fronts at once.</t>
         </is>
       </c>
       <c r="E22" s="36" t="inlineStr">
         <is>
-          <t>Arms routes, sponsors, and displaced administrations are carrying the crisis across borders. Civilian relief and armed support now demand separate choices.</t>
+          <t>Arms routes and foreign sponsors are carrying the crisis across borders. Civilian relief and armed support demand separate choices. The fighting sides are reorganizing their supplies, defenses and mobile columns. In a few units, night gatherings, sworn oaths and repeated signs have appeared that no one outside their ranks can explain.</t>
         </is>
       </c>
       <c r="F22" s="37" t="inlineStr">
@@ -3374,7 +3374,7 @@
       <c r="L24" s="54" t="n"/>
       <c r="M24" s="72" t="inlineStr">
         <is>
-          <t>To Be Reworked</t>
+          <t>Needs Testing</t>
         </is>
       </c>
     </row>
@@ -3491,12 +3491,12 @@
       </c>
       <c r="C27" s="30" t="inlineStr">
         <is>
-          <t>A Friday clearance sale draws crowds into shops across the world. Quartermasters, intelligence officers, and ministry clerks join the rush, bringing government orders to counters already piled with civilian purchases.</t>
+          <t>A Friday clearance sale draws crowds into shops across the world. Quartermasters, staff officers, and ministry clerks join the rush, bringing government orders to counters already piled with civilian purchases.\n\nBase-game national decisions, guarantees, intelligence operations, license purchases, military-industrial organizations, equipment upgrades, leader promotions, leader traits, preferred tactics, and special projects keep their normal price.</t>
         </is>
       </c>
       <c r="D27" s="35" t="inlineStr">
         <is>
-          <t>If this evolution is enabled and chaos is at least [?constant:black_friday_event.evolution_chaos|0] when the sale begins, eligible purchases receive [?constant:black_friday_event.evolution_discount_percent|0]% off. That rate lasts until the next daily tick, even if chaos falls.</t>
+          <t>If this evolution is enabled and chaos is at least 600 when the sale begins, eligible purchases receive 75% off. That rate lasts for the rest of the day, even if chaos falls.</t>
         </is>
       </c>
       <c r="E27" s="36" t="n"/>

</xml_diff>

<commit_message>
Align the event catalog names with the localised event names and describe Events 22 and 54 as in game
32 Events-sheet names now equal the event registry names, including Events 22, 46, 84 and 85, and the matching Cluster Memberships display names follow. Event 22 Details uses the Concentration Camps Event Details text. Event 54 gets its own Event Details entry in game, and the sheet repeats it; CSV exports regenerated.
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -3294,12 +3294,12 @@
       </c>
       <c r="B23" s="30" t="inlineStr">
         <is>
-          <t>Spain Antisemitism</t>
+          <t>Concentration Camps</t>
         </is>
       </c>
       <c r="C23" s="30" t="inlineStr">
         <is>
-          <t>A violent antisemitic faction emerges during the Spanish Civil War, seeks an alliance with Nazi Germany, and threatens Jewish communities across Europe.</t>
+          <t>A government with occupied regions, active resistance or a list of political enemies opens detention camps in about a fifth of its states. The camps hold people without trial, and many of them die of hunger, disease and overwork. Neighbours hear reports and the prisoners' families begin to search. The country can close the camps, review the cases, put the prisoners to work or widen the network.</t>
         </is>
       </c>
       <c r="D23" s="35" t="n"/>
@@ -3431,7 +3431,7 @@
       </c>
       <c r="B26" s="30" t="inlineStr">
         <is>
-          <t>Alien technology in Antarctica</t>
+          <t>Alien Technology in Antarctica</t>
         </is>
       </c>
       <c r="C26" s="30" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="B42" s="30" t="inlineStr">
         <is>
-          <t>Disease in divisions</t>
+          <t>Disease in Divisions</t>
         </is>
       </c>
       <c r="C42" s="30" t="inlineStr">
@@ -4320,7 +4320,7 @@
       </c>
       <c r="B44" s="30" t="inlineStr">
         <is>
-          <t>Massive flood</t>
+          <t>Massive Flood</t>
         </is>
       </c>
       <c r="C44" s="30" t="inlineStr">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="B45" s="30" t="inlineStr">
         <is>
-          <t>Space race</t>
+          <t>Space Race</t>
         </is>
       </c>
       <c r="C45" s="30" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="B46" s="30" t="inlineStr">
         <is>
-          <t>Third Balkan war</t>
+          <t>Third Balkan War</t>
         </is>
       </c>
       <c r="C46" s="30" t="inlineStr">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="B47" s="30" t="inlineStr">
         <is>
-          <t>Seismic Archive</t>
+          <t>Unknown Event</t>
         </is>
       </c>
       <c r="C47" s="30" t="inlineStr">
@@ -4470,7 +4470,7 @@
       </c>
       <c r="B48" s="30" t="inlineStr">
         <is>
-          <t>BOOM</t>
+          <t>Boom!</t>
         </is>
       </c>
       <c r="C48" s="30" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="B53" s="30" t="inlineStr">
         <is>
-          <t>Intel Leaked</t>
+          <t>Intelligence Leak</t>
         </is>
       </c>
       <c r="C53" s="30" t="inlineStr">
@@ -4740,7 +4740,7 @@
       </c>
       <c r="C55" s="30" t="inlineStr">
         <is>
-          <t>A country enters a sudden infrastructure boom.</t>
+          <t>A breakthrough reaches the world's laboratories almost at once. Engineers in every country are suddenly working from the same new design, and ministries begin planning how to build it at scale for industry and the armed forces.</t>
         </is>
       </c>
       <c r="D55" s="35" t="n"/>
@@ -4774,7 +4774,7 @@
       </c>
       <c r="B56" s="30" t="inlineStr">
         <is>
-          <t>The Great Infrastructure Project</t>
+          <t>Great Infrastructure Project</t>
         </is>
       </c>
       <c r="C56" s="30" t="inlineStr">
@@ -4813,7 +4813,7 @@
       </c>
       <c r="B57" s="30" t="inlineStr">
         <is>
-          <t>The Navy</t>
+          <t>Navy</t>
         </is>
       </c>
       <c r="C57" s="30" t="inlineStr">
@@ -4852,7 +4852,7 @@
       </c>
       <c r="B58" s="30" t="inlineStr">
         <is>
-          <t>The Radar</t>
+          <t>Radars</t>
         </is>
       </c>
       <c r="C58" s="30" t="inlineStr">
@@ -4930,7 +4930,7 @@
       </c>
       <c r="B60" s="30" t="inlineStr">
         <is>
-          <t>AI focus aggressive</t>
+          <t>AI Focus Aggressive</t>
         </is>
       </c>
       <c r="C60" s="30" t="inlineStr">
@@ -5086,7 +5086,7 @@
       </c>
       <c r="B64" s="30" t="inlineStr">
         <is>
-          <t>End Subject Status</t>
+          <t>Subject Independence</t>
         </is>
       </c>
       <c r="C64" s="30" t="inlineStr">
@@ -5125,7 +5125,7 @@
       </c>
       <c r="B65" s="30" t="inlineStr">
         <is>
-          <t>Border fortifications</t>
+          <t>Border Forts</t>
         </is>
       </c>
       <c r="C65" s="30" t="inlineStr">
@@ -5360,7 +5360,7 @@
       </c>
       <c r="B72" s="30" t="inlineStr">
         <is>
-          <t>Persia</t>
+          <t>Persian Empire</t>
         </is>
       </c>
       <c r="C72" s="30" t="inlineStr">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="B73" s="30" t="inlineStr">
         <is>
-          <t>Ireland reclaims North</t>
+          <t>Ireland Reclaims North</t>
         </is>
       </c>
       <c r="C73" s="30" t="inlineStr">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="B74" s="30" t="inlineStr">
         <is>
-          <t>Mongols rise</t>
+          <t>Mongols Rise</t>
         </is>
       </c>
       <c r="C74" s="30" t="inlineStr">
@@ -5500,7 +5500,7 @@
       </c>
       <c r="B76" s="30" t="inlineStr">
         <is>
-          <t>Tannu Tuva joins a faction</t>
+          <t>Tannu Tuva Joins Allies</t>
         </is>
       </c>
       <c r="C76" s="30" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="B77" s="30" t="inlineStr">
         <is>
-          <t>USA tests weapons</t>
+          <t>USA Tests Weapons</t>
         </is>
       </c>
       <c r="C77" s="30" t="inlineStr">
@@ -5570,7 +5570,7 @@
       </c>
       <c r="B78" s="30" t="inlineStr">
         <is>
-          <t>Eq aid</t>
+          <t>Equipment Aid</t>
         </is>
       </c>
       <c r="C78" s="30" t="inlineStr">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="B79" s="30" t="inlineStr">
         <is>
-          <t>Border Conflict</t>
+          <t>Border War</t>
         </is>
       </c>
       <c r="C79" s="30" t="inlineStr">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="B82" s="30" t="inlineStr">
         <is>
-          <t>British tax</t>
+          <t>England Tax</t>
         </is>
       </c>
       <c r="C82" s="30" t="inlineStr">
@@ -5780,7 +5780,7 @@
       </c>
       <c r="B84" s="30" t="inlineStr">
         <is>
-          <t>Agency upgrade</t>
+          <t>Agency Upgrade</t>
         </is>
       </c>
       <c r="C84" s="30" t="inlineStr">
@@ -5815,7 +5815,7 @@
       </c>
       <c r="B85" s="30" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>Political Power</t>
         </is>
       </c>
       <c r="C85" s="30" t="inlineStr">
@@ -5850,7 +5850,7 @@
       </c>
       <c r="B86" s="30" t="inlineStr">
         <is>
-          <t>XP</t>
+          <t>Experience</t>
         </is>
       </c>
       <c r="C86" s="30" t="inlineStr">
@@ -5920,7 +5920,7 @@
       </c>
       <c r="B88" s="30" t="inlineStr">
         <is>
-          <t>It’s WW1</t>
+          <t>The First World War</t>
         </is>
       </c>
       <c r="C88" s="30" t="inlineStr">
@@ -5955,7 +5955,7 @@
       </c>
       <c r="B89" s="30" t="inlineStr">
         <is>
-          <t>Mines everywhere</t>
+          <t>Mines</t>
         </is>
       </c>
       <c r="C89" s="30" t="inlineStr">
@@ -5990,7 +5990,7 @@
       </c>
       <c r="B90" s="30" t="inlineStr">
         <is>
-          <t>Tech sharing</t>
+          <t>Tech Sharing Group</t>
         </is>
       </c>
       <c r="C90" s="30" t="inlineStr">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="B91" s="30" t="inlineStr">
         <is>
-          <t>Suicide craft</t>
+          <t>Kamikaze</t>
         </is>
       </c>
       <c r="C91" s="30" t="inlineStr">
@@ -6169,7 +6169,7 @@
       </c>
       <c r="B95" s="30" t="inlineStr">
         <is>
-          <t>Half gone</t>
+          <t>Half Gone</t>
         </is>
       </c>
       <c r="C95" s="30" t="inlineStr">
@@ -6204,7 +6204,7 @@
       </c>
       <c r="B96" s="30" t="inlineStr">
         <is>
-          <t>Occupation revolt</t>
+          <t>Occupation Revolt</t>
         </is>
       </c>
       <c r="C96" s="30" t="inlineStr">
@@ -22213,7 +22213,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Third Balkan war</t>
+          <t>Third Balkan War</t>
         </is>
       </c>
       <c r="F9" s="54" t="inlineStr">
@@ -22387,7 +22387,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Subjects Break Free</t>
+          <t>Subject Independence</t>
         </is>
       </c>
       <c r="F15" s="54" t="inlineStr">
@@ -22499,7 +22499,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>The Offensive</t>
+          <t>AI Focus Aggressive</t>
         </is>
       </c>
       <c r="F19" s="54" t="inlineStr">
@@ -23085,7 +23085,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>The Great Infrastructure Project</t>
+          <t>Great Infrastructure Project</t>
         </is>
       </c>
       <c r="F39" s="54" t="inlineStr">
@@ -23112,7 +23112,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>The Black Market</t>
+          <t>Radars</t>
         </is>
       </c>
       <c r="F40" s="54" t="inlineStr">
@@ -23193,7 +23193,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Intel Leaked</t>
+          <t>Intelligence Leak</t>
         </is>
       </c>
       <c r="F43" s="54" t="inlineStr">
@@ -23498,7 +23498,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>BOOM</t>
+          <t>Boom!</t>
         </is>
       </c>
       <c r="F54" s="54" t="inlineStr">
@@ -23633,7 +23633,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>The Great Shuffle</t>
+          <t>Unknown Event</t>
         </is>
       </c>
       <c r="F59" s="54" t="inlineStr">
@@ -23771,7 +23771,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>The Navy</t>
+          <t>Navy</t>
         </is>
       </c>
       <c r="F65" s="54" t="inlineStr">
@@ -23802,7 +23802,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>Border Fortifications</t>
+          <t>Border Forts</t>
         </is>
       </c>
       <c r="F66" s="54" t="inlineStr">
@@ -23918,7 +23918,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>Subjects Break Free</t>
+          <t>Subject Independence</t>
         </is>
       </c>
       <c r="F70" s="54" t="inlineStr">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>Monsters from the Deep</t>
+          <t>Massive Flood</t>
         </is>
       </c>
       <c r="F71" s="54" t="inlineStr">
@@ -24052,7 +24052,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>The Navy</t>
+          <t>Navy</t>
         </is>
       </c>
       <c r="F76" s="54" t="inlineStr">
@@ -24083,7 +24083,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>Border Fortifications</t>
+          <t>Border Forts</t>
         </is>
       </c>
       <c r="F77" s="54" t="inlineStr">

</xml_diff>

<commit_message>
Event catalog: mirror Events 22, 30 and 40 in-game text and implementation
Event 22 gets Evo I to III bodies, type Minor Repeatable, cluster 16 Domestic Unrest as Severe member (removed from Military Preparation). Event 30 gets the in-game Details and the two implemented evolution rows, stale Evo IV text cleared. Event 40 gets Details and Evo I to III, type Minor Fire-Once. All three use Needs Testing. CSV exports regenerated.
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -3302,15 +3302,27 @@
           <t>A government with occupied regions, active resistance or a list of political enemies opens detention camps in about a fifth of its states. The camps hold people without trial, and many of them die of hunger, disease and overwork. Neighbours hear reports and the prisoners' families begin to search. The country can close the camps, review the cases, put the prisoners to work or widen the network.</t>
         </is>
       </c>
-      <c r="D23" s="35" t="n"/>
-      <c r="E23" s="36" t="n"/>
-      <c r="F23" s="37" t="n"/>
+      <c r="D23" s="35" t="inlineStr">
+        <is>
+          <t>Part of the camp network receives a different purpose and chain of command. Killing orders replace detention and forced labour in selected camps, and the government that receives them has to decide whether to accept.</t>
+        </is>
+      </c>
+      <c r="E23" s="36" t="inlineStr">
+        <is>
+          <t>Rations are cut and transports run full across the whole network at once. Deaths in every state that holds a camp rise far above the usual figure for a month, and families begin to count the missing.</t>
+        </is>
+      </c>
+      <c r="F23" s="37" t="inlineStr">
+        <is>
+          <t>The network spreads until it touches about half of the states, with detention camps and killing camps side by side. Another synchronized wave of deaths follows, and the camps become an emergency for the whole government.</t>
+        </is>
+      </c>
       <c r="G23" s="38" t="n"/>
       <c r="H23" s="39" t="n"/>
       <c r="I23" s="40" t="n"/>
-      <c r="J23" s="65" t="inlineStr">
-        <is>
-          <t>Minor Fire-Once</t>
+      <c r="J23" s="67" t="inlineStr">
+        <is>
+          <t>Minor Repeatable</t>
         </is>
       </c>
       <c r="K23" s="54" t="n">
@@ -3318,12 +3330,12 @@
       </c>
       <c r="L23" s="54" t="inlineStr">
         <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="M23" s="72" t="inlineStr">
-        <is>
-          <t>To Be Reworked</t>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="M23" s="70" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
         </is>
       </c>
     </row>
@@ -3675,21 +3687,21 @@
       </c>
       <c r="C31" s="30" t="inlineStr">
         <is>
-          <t>A time traveler known as “Time Traveler” advises a country and warns certain governments against wars that history says they will lose. A later route can bring Napoleon back, followed by a robot invasion from the future.</t>
+          <t>A man who remembers a later time appears in one country and proves it with a page of secrets and a forecast that comes true. The government chooses how he works with the state, and each piece of advice he gives must be carried out before it pays. Foreign services copy his records, plant forgeries, offer him asylum and try to take him. The more the world acts on what he says, the less his memory of the future describes it.</t>
         </is>
       </c>
       <c r="D31" s="82" t="inlineStr">
         <is>
-          <t>Time Traveler: a historical warning system guides governments away from wars that history says they will lose.</t>
-        </is>
-      </c>
-      <c r="E31" s="36" t="n"/>
+          <t>What the visitor knows about the careers and failures of the people around him becomes a political force. The government decides whether he stays an adviser, receives emergency authority, takes office, is arrested, leaves or disappears, and the ministries, the officers and the experts choose their sides.</t>
+        </is>
+      </c>
+      <c r="E31" s="36" t="inlineStr">
+        <is>
+          <t>People from earlier centuries begin to appear in the modern world. Each one has a name that millions still know, a claim on the loyalty of some and the fear of others, and no knowledge of the century they have arrived in. Governments must decide what to make of them before others do.</t>
+        </is>
+      </c>
       <c r="F31" s="37" t="n"/>
-      <c r="G31" s="85" t="inlineStr">
-        <is>
-          <t>Napoleon returns (Pretzel Logic), World End scenario: army of robots from the future invade, basically like in the movie Terminator.</t>
-        </is>
-      </c>
+      <c r="G31" s="85" t="n"/>
       <c r="H31" s="39" t="n"/>
       <c r="I31" s="40" t="n"/>
       <c r="J31" s="66" t="inlineStr">
@@ -3701,9 +3713,9 @@
         <v>1</v>
       </c>
       <c r="L31" s="54" t="n"/>
-      <c r="M31" s="72" t="inlineStr">
-        <is>
-          <t>To Be Reworked</t>
+      <c r="M31" s="70" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
         </is>
       </c>
     </row>
@@ -4200,27 +4212,39 @@
       </c>
       <c r="C41" s="30" t="inlineStr">
         <is>
-          <t>A random Arabian country falls under British control through a Lawrence of Arabia intervention.</t>
-        </is>
-      </c>
-      <c r="D41" s="35" t="n"/>
-      <c r="E41" s="36" t="n"/>
-      <c r="F41" s="37" t="n"/>
+          <t>Britain recalls T. E. Lawrence, reported dead after a motorcycle crash, and sends him into one Arabian government that is weak, useful or willing to bargain. The government decides how far the mission may go, officers and ministries take sides, and Britain pays for every shipment in real equipment. Each government ends in a settlement of its own, from a protectorate to an alliance, an armed partnership, a quiet withdrawal or an expulsion. Later governments follow after months of delay and remember what happened to the ones before.</t>
+        </is>
+      </c>
+      <c r="D41" s="35" t="inlineStr">
+        <is>
+          <t>British money and arms reach smugglers, officers, railway workers, couriers and local leaders. Their cells can sabotage a line, divide a garrison or demand a new government.</t>
+        </is>
+      </c>
+      <c r="E41" s="36" t="inlineStr">
+        <is>
+          <t>Governments that accepted British help begin to act as one order. Their officers train together, their ports serve the same convoys and their ministers write to each other. Each can contribute, bargain, refuse or turn against the arrangement.</t>
+        </is>
+      </c>
+      <c r="F41" s="37" t="inlineStr">
+        <is>
+          <t>Partners, allies and independent governments are drawn towards one federation. It can become a British dominion, a sovereign union or a state built around Lawrence himself.</t>
+        </is>
+      </c>
       <c r="G41" s="38" t="n"/>
       <c r="H41" s="39" t="n"/>
       <c r="I41" s="40" t="n"/>
-      <c r="J41" s="67" t="inlineStr">
-        <is>
-          <t>Minor Repeatable</t>
+      <c r="J41" s="65" t="inlineStr">
+        <is>
+          <t>Minor Fire-Once</t>
         </is>
       </c>
       <c r="K41" s="54" t="n">
         <v>1</v>
       </c>
       <c r="L41" s="54" t="n"/>
-      <c r="M41" s="72" t="inlineStr">
-        <is>
-          <t>To Be Reworked</t>
+      <c r="M41" s="70" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
         </is>
       </c>
     </row>
@@ -21728,12 +21752,12 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>1, 6, 31, 63</t>
+          <t>1, 6, 22, 31, 63</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Medium, High, Medium, Medium</t>
+          <t>Medium, High, Severe, Medium, Medium</t>
         </is>
       </c>
       <c r="F17" s="69" t="inlineStr">
@@ -21804,12 +21828,12 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>22, 42, 56, 64</t>
+          <t>42, 56, 64</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>High, Low, Medium, Medium</t>
+          <t>Low, Medium, Medium</t>
         </is>
       </c>
       <c r="F19" s="69" t="inlineStr">
@@ -23884,19 +23908,19 @@
         </is>
       </c>
       <c r="C69" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D69" s="5" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>Random Terror</t>
+          <t>Concentration Camps</t>
         </is>
       </c>
       <c r="F69" s="54" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Severe</t>
         </is>
       </c>
       <c r="G69" s="5" t="n"/>
@@ -23911,14 +23935,14 @@
         </is>
       </c>
       <c r="C70" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D70" s="5" t="n">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>Subject Independence</t>
+          <t>Random Terror</t>
         </is>
       </c>
       <c r="F70" s="54" t="inlineStr">
@@ -23926,62 +23950,62 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="G70" s="5" t="inlineStr">
-        <is>
-          <t>Also Liberations at Medium severity.</t>
-        </is>
-      </c>
+      <c r="G70" s="5" t="n"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>Alien Invasions</t>
+          <t>Domestic Unrest</t>
         </is>
       </c>
       <c r="C71" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D71" s="5" t="n">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>Massive Flood</t>
+          <t>Subject Independence</t>
         </is>
       </c>
       <c r="F71" s="54" t="inlineStr">
         <is>
-          <t>Severe</t>
-        </is>
-      </c>
-      <c r="G71" s="5" t="n"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>Also Liberations at Medium severity.</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Military Preparation</t>
+          <t>Alien Invasions</t>
         </is>
       </c>
       <c r="C72" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D72" s="5" t="n">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>Concentration Camps</t>
+          <t>Massive Flood</t>
         </is>
       </c>
       <c r="F72" s="54" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Severe</t>
         </is>
       </c>
       <c r="G72" s="5" t="n"/>

</xml_diff>

<commit_message>
Align the event catalog with restored historical localisation
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -2615,7 +2615,7 @@
       </c>
       <c r="D11" s="82" t="inlineStr">
         <is>
-          <t>Ships stop arriving from a second island. Nobody yet knows it is lost, but its neighbors have noticed the silence.</t>
+          <t xml:space="preserve">Death reaches a second island and empties it slowly enough to resemble lost shipping or an abandoned harbor. The silence spreads from shore to shore while mainland governments remain uncertain of its cause.</t>
         </is>
       </c>
       <c r="E11" s="83" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="C12" s="30" t="inlineStr">
         <is>
-          <t>Strangers keep meeting in the wrong places. Couriers vanish, equipment fails, and the same quiet methods turn up in distant incidents. Nobody can say who is behind them.</t>
+          <t xml:space="preserve">Strangers keep meeting in the wrong places. Couriers vanish, equipment fails, and the same quiet methods turn up in distant incidents. Following the trail can expose the pattern, while practical precautions may blunt the next attack.</t>
         </is>
       </c>
       <c r="D12" s="82" t="inlineStr">
@@ -2915,12 +2915,12 @@
       </c>
       <c r="G16" s="85" t="inlineStr">
         <is>
-          <t>The manifesto now shapes regional politics. Governments invoke it to seek aid, defend local charters, resist threats, or ask for association, and small states must decide whether the commonwealth is a refuge, a useful partner, or an ambitious neighbor.</t>
+          <t xml:space="preserve">The Manifesto shapes regional politics. Governments invoke it when seeking aid, defending local charters, resisting threats, or seeking association. Small states must decide whether the commonwealth is a refuge, a useful partner, or an ambitious neighbor.</t>
         </is>
       </c>
       <c r="H16" s="86" t="inlineStr">
         <is>
-          <t>The world around the commonwealth is coming apart. Harbors, trains, fortifications, and refuge towns all need the same stores. Citizens and League members ask whether the gates will protect them, who must serve inside, and which neighbors will share the burden.</t>
+          <t xml:space="preserve">The world around the commonwealth is coming apart. Harbors, trains, fortifications, and refuge towns all need the same stores. Citizens and league members ask whether the gates will protect them, who must serve inside, and which neighbors will share the burden.</t>
         </is>
       </c>
       <c r="I16" s="40" t="n"/>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="D20" s="82" t="inlineStr">
         <is>
-          <t>The soldiers from nowhere have district staffs, proper rolls, and officers the government can actually hold responsible.</t>
+          <t xml:space="preserve">The soldiers from nowhere now have district staffs, proper rolls, and officers the government can actually hold responsible.</t>
         </is>
       </c>
       <c r="E20" s="83" t="inlineStr">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="B24" s="30" t="inlineStr">
         <is>
-          <t>Soviet Nuclear Bombs</t>
+          <t xml:space="preserve">SOV Nuclear Bombs</t>
         </is>
       </c>
       <c r="C24" s="30" t="inlineStr">
@@ -3687,7 +3687,7 @@
       </c>
       <c r="C31" s="30" t="inlineStr">
         <is>
-          <t>A man who remembers a later time appears in one country and proves it with a page of secrets and a forecast that comes true. The government chooses how he works with the state, and each piece of advice he gives must be carried out before it pays. Foreign services copy his records, plant forgeries, offer him asylum and try to take him. The more the world acts on what he says, the less his memory of the future describes it.</t>
+          <t xml:space="preserve">A man who remembers a later time appears in one country and proves it with a page of secrets and a forecast that comes true. The government chooses how he works with the state, and each piece of advice he gives must be carried out before its reward is paid. Foreign services copy his records, plant forgeries, offer him asylum and try to take him. The more the world acts on what he says, the less his memory of the future still describes it. Officials who depend on him begin to fight over him and the country that holds him may split, and as the order of the world loosens people from earlier centuries start to arrive.</t>
         </is>
       </c>
       <c r="D31" s="82" t="inlineStr">
@@ -3795,12 +3795,12 @@
       </c>
       <c r="C33" s="30" t="inlineStr">
         <is>
-          <t>Missile programs have spread across the world. Countries can build and harden launch sites, stock operational missiles, improve guidance, and secure the officers and codes that control them. Heavier arsenals, guidance failures, special warheads, rogue commands, and automatic retaliation can transform the crisis.</t>
+          <t xml:space="preserve">Missile programmes have spread across the world. Countries can build and harden launch sites, stock operational missiles, improve guidance, and secure the officers and codes that control them. Heavier arsenals, guidance failures, special warheads, rogue commands, and automatic retaliation can transform the crisis.</t>
         </is>
       </c>
       <c r="D33" s="35" t="inlineStr">
         <is>
-          <t>Countries with working launch sites and enough industry can adopt a saturation doctrine for massed salvos. Saturation attacks can overwhelm defenses, but they consume many missiles and strain readiness and command control.</t>
+          <t xml:space="preserve">Countries with working launch sites and enough industry can adopt a saturation doctrine for massed salvos. Saturation attacks can overwhelm defences, but they consume many missiles and strain readiness and command control.</t>
         </is>
       </c>
       <c r="E33" s="36" t="inlineStr">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="F33" s="37" t="inlineStr">
         <is>
-          <t>Countries that already possess chemical, biological, nuclear, or thermonuclear weapons can adapt them for missile delivery. Each launch still requires an authorized warhead held in secure custody.</t>
+          <t xml:space="preserve">Countries that already possess chemical, biological, nuclear, or thermonuclear weapons can adapt them for missile delivery. Each launch still requires an authorised warhead held in secure custody.</t>
         </is>
       </c>
       <c r="G33" s="38" t="inlineStr">
@@ -3865,7 +3865,7 @@
       </c>
       <c r="F34" s="37" t="inlineStr">
         <is>
-          <t>Global Acid Rain: The fronts merge into a worldwide layer that exposes every inhabited state in its path and produces regional superstorms with nine-day forecasts.</t>
+          <t xml:space="preserve">Global Acid Rain: The fronts merge into a worldwide layer that exposes every valid inhabited state and produces regional superstorms with nine-day forecasts.</t>
         </is>
       </c>
       <c r="G34" s="38" t="n"/>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="B55" s="30" t="inlineStr">
         <is>
-          <t>New Technology</t>
+          <t xml:space="preserve">Random Tech</t>
         </is>
       </c>
       <c r="C55" s="30" t="inlineStr">
@@ -4915,7 +4915,7 @@
       </c>
       <c r="B59" s="30" t="inlineStr">
         <is>
-          <t>Industrial Complexes</t>
+          <t xml:space="preserve">Free Civs</t>
         </is>
       </c>
       <c r="C59" s="30" t="inlineStr">
@@ -5032,7 +5032,7 @@
       </c>
       <c r="B62" s="30" t="inlineStr">
         <is>
-          <t>Arms Factory Conversion</t>
+          <t xml:space="preserve">Mils into Civs</t>
         </is>
       </c>
       <c r="C62" s="30" t="inlineStr">
@@ -5188,7 +5188,7 @@
       </c>
       <c r="B66" s="30" t="inlineStr">
         <is>
-          <t>Random Leader Trait</t>
+          <t xml:space="preserve">Random Trait</t>
         </is>
       </c>
       <c r="C66" s="30" t="inlineStr">
@@ -5223,7 +5223,7 @@
       </c>
       <c r="B67" s="30" t="inlineStr">
         <is>
-          <t>Construction Industrial Capacity</t>
+          <t xml:space="preserve">CIC</t>
         </is>
       </c>
       <c r="C67" s="30" t="inlineStr">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="B75" s="30" t="inlineStr">
         <is>
-          <t>Japan in California</t>
+          <t xml:space="preserve">Japan California</t>
         </is>
       </c>
       <c r="C75" s="30" t="inlineStr">
@@ -5769,7 +5769,7 @@
       </c>
       <c r="B83" s="30" t="inlineStr">
         <is>
-          <t>Step Toward Mobilization</t>
+          <t xml:space="preserve">Law Upgrade</t>
         </is>
       </c>
       <c r="C83" s="30" t="inlineStr">
@@ -6158,7 +6158,7 @@
       </c>
       <c r="B94" s="30" t="inlineStr">
         <is>
-          <t>Portugal Demands Galicia</t>
+          <t xml:space="preserve">Portugal Galicia</t>
         </is>
       </c>
       <c r="C94" s="30" t="inlineStr">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" s="30" t="inlineStr">
         <is>
-          <t>Division Templates Locked</t>
+          <t xml:space="preserve">Divisions Lock</t>
         </is>
       </c>
       <c r="C97" s="30" t="inlineStr">
@@ -21177,7 +21177,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Sudden wars and armed conflicts break out between countries, turning local disputes, opportunistic attacks, internal fractures, and alliance betrayals into wider fighting.</t>
+          <t xml:space="preserve">Sudden wars and armed conflicts break out between countries, turning local disputes, opportunistic attacks, and border shocks into a wider chain of fighting.</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -21248,12 +21248,12 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Diplomacy</t>
+          <t xml:space="preserve">Diplomatic Panic</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>International relations destabilize through diplomatic crises, faction pressure, treaties, strategic alignment, aggressive posturing, and intervention.</t>
+          <t xml:space="preserve">Diplomatic crises spread through public quarrels, collapsing relations, hurried guarantees, and minor states pressed to choose among nearby blocs.</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -21367,7 +21367,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Countries revive, construct, or transform into major historical, religious, imperial, or alternative political formations. The Formables cluster remains repeatable; Africa Is One is its Severe Event 12 member, a tier-4 Minor Fire-Once entry with entry event chaosx.nr12.1.</t>
+          <t xml:space="preserve">Formables gather negotiated restoration and union projects. Africa Is One builds a protection-first Charter League through aid, guarantees, liberation recognition, consent, constitutional routes, and rival settlements. The Formables cluster remains repeatable; Africa Is One is its Severe Event 12 member, a tier-4 Minor Fire-Once entry with entry event chaosx.nr12.1.</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -21633,7 +21633,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Disease outbreaks and biological crises spread through countries, armies, and populations, creating escalating health and military emergencies.</t>
+          <t xml:space="preserve">Severe outbreaks establish persistent conditions in affected states. Each disease follows its own transmission routes and demands material, military, and time investment to contain it.</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -22431,7 +22431,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Diplomacy</t>
+          <t xml:space="preserve">Diplomatic Panic</t>
         </is>
       </c>
       <c r="C16" s="5" t="n">
@@ -22458,7 +22458,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Diplomacy</t>
+          <t xml:space="preserve">Diplomatic Panic</t>
         </is>
       </c>
       <c r="C17" s="5" t="n">
@@ -22485,7 +22485,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Diplomacy</t>
+          <t xml:space="preserve">Diplomatic Panic</t>
         </is>
       </c>
       <c r="C18" s="5" t="n">
@@ -22512,7 +22512,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Diplomacy</t>
+          <t xml:space="preserve">Diplomatic Panic</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
@@ -22678,7 +22678,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Arms Factory Conversion</t>
+          <t xml:space="preserve">Mils into Civs</t>
         </is>
       </c>
       <c r="F24" s="54" t="inlineStr">
@@ -23163,7 +23163,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Industrial Complexes</t>
+          <t xml:space="preserve">Free Civs</t>
         </is>
       </c>
       <c r="F41" s="54" t="inlineStr">
@@ -23275,7 +23275,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>New Technology</t>
+          <t xml:space="preserve">Random Tech</t>
         </is>
       </c>
       <c r="F45" s="54" t="inlineStr">
@@ -23302,7 +23302,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Random Leader Trait</t>
+          <t xml:space="preserve">Random Trait</t>
         </is>
       </c>
       <c r="F46" s="54" t="inlineStr">
@@ -24307,8 +24307,8 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Pact: Turns eligible minor governments into dispersed Fury states and organizes them into the Fury Pact. Higher intensity spreads the pact farther across the world and strengthens its opening forces.
-Hostile: Turns eligible minor governments into dispersed hostile Fury states that immediately pursue neighboring wars. Higher intensity spreads the Fury farther across the world and strengthens their opening attacks.</t>
+          <t xml:space="preserve">Pact: Turns eligible non-player minor countries into dispersed Fury actors and organizes them into the Fury Pact. Higher intensity spreads more Fury states across the world and grants stronger evolved openings.
+Hostile: Turns eligible non-player minor countries into dispersed hostile Fury actors that immediately pursue neighboring wars. Higher intensity spreads more Fury states across the world and escalates their opening pressure.</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -24407,14 +24407,14 @@
       </c>
       <c r="C8" s="52" t="inlineStr">
         <is>
-          <t>Sovereign Scatter: Every viable independence movement breaks away. Hosts keep a protected remnant, each new state gets its own starting territory, and none joins a league or faction. Intensity changes territory, forces, and pressure.
-Open Congress: Every viable independence movement breaks away from a protected host. The new states join an informal congress, and higher intensity strengthens its charter and shared reserve.
-Separation Wars: Every viable independence movement breaks away. A new state able to confront its former host may open one war of separation. The others receive a regional threat mission.
-Host Wars: Every viable independence movement breaks away. Each new state may open one war against its former host. Hosts keep their homelands, and wars that cannot start become regional threat missions.
-Neighbor Wars: Every viable independence movement breaks away. Each new state may open one war against a neighboring state released in the same crisis. Each state is targeted once, so no all-against-all cascade follows.
-Outsider Wars: Every viable independence movement breaks away. Each new state may open one war against a nearby independent state outside the League and every faction. Each target is chosen once and distance keeps the crisis regional.
-Patron Worlds: Every viable independence movement breaks away. Each new state seeks one reachable major patron, favoring shared ideology and regional proximity. Intensity scales influence, aid, and recognition.
-Great Partition: Every viable independence movement breaks away. Each host keeps one protected remnant, preferring its capital, then a safe core state. Higher intensity adds the next tier of territory, border pressure, claims, and ambitions.</t>
+          <t xml:space="preserve">Sovereign Scatter: Every viable movement is attempted. Each release keeps a protected former-host remnant and unique anchor. States remain outside pre-formed leagues and retain no release-created faction ties. Intensity changes territory, forces, institutions, and pressure.
+Open Congress: Every viable movement is attempted under protected hosts and unique anchors. New states join an informal congress network. Higher intensity strengthens its charter and shared reserve.
+Separation Wars: Every viable movement is attempted. A country that can lawfully confront its surviving former host may open one separation war. Others receive a regional threat mission.
+Host Wars: Every viable movement is attempted. Each new country may face one bounded former-host conflict. Invalid declarations become regional threat missions. Host remnants and homelands are secured first.
+Neighbor Wars: Every viable movement is attempted. Each new country may open one bounded war against one neighboring release from the same incident. One-time targets prevent an all-against-all cascade.
+Outsider Wars: Every viable movement is attempted. Each new country may open one bounded war against one nearby independent state outside the League and every faction. Distance and one-time targets keep the crisis regional.
+Patron Worlds: Every viable movement is attempted. Each new country seeks one reachable major patron, preferring ideological affinity and regional proximity. Intensity scales influence, aid, recognition, and capacity.
+Great Partition: Every viable movement is attempted. Hosts retain one protected remnant state, preferring a controlled capital, then a safe core or owned state. Intensity grants the next non-overlapping tier, with stronger border pressure, host claims, ambitions, and formables.</t>
         </is>
       </c>
       <c r="D8" s="52" t="inlineStr">
@@ -24424,10 +24424,10 @@
       </c>
       <c r="E8" s="52" t="inlineStr">
         <is>
-          <t>Low: Each release gets only its starting territory, fragile defenses, scarce stocks, weak institutions, low recognition, and severe instability.
-Medium: Releases receive compact territory, militia and border formations, baseline institutions, and ordinary route access.
-High: Releases receive wider territory where borders allow, armed forces, stronger depots and officers, firmer institutions, and faster ambitions.
-Maximum: Releases receive the largest territory and forces, rare support where their route allows it, high-chaos access, early formable discovery, and aggressive AI.</t>
+          <t xml:space="preserve">Low: All viable candidates are still attempted. Each valid release receives only its anchor, fragile local defense, scarce stocks, weak institutions, low recognition, and severe opening instability.
+Medium: All viable candidates are still attempted. Valid releases receive compact territory, viable militia and border formations, baseline institutions, and ordinary route access.
+High: All viable candidates are still attempted. Valid releases receive extended territory where collisions permit, armed forces, stronger depots and officers, firmer institutions, faster league development, and accelerated ambitions.
+Maximum: All viable candidates are still attempted. Valid releases receive the strongest non-overlapping territory and forces, rare support where their researched route permits it, high-chaos access, early formable discovery, and aggressive AI pressure.</t>
         </is>
       </c>
       <c r="F8" s="76" t="inlineStr">
@@ -24527,7 +24527,7 @@
       </c>
       <c r="C11" s="54" t="inlineStr">
         <is>
-          <t>Africa Is One: Unites Africa under a powerful continental state, establishes the Charter League and its regional institutions, and prepares the wars required to complete unification.
+          <t xml:space="preserve">Africa Is One: Forms a strong Africa, opens the Charter League, regional authority, Authority Atlas, sponsor, proof-ledger, and post-unification systems, then opens the continental unification war office.
 World Is One: Forms Africa and prepares the World Is One final campaign. Rival continental powers become eligible for treaties, containment, or war, while the proclamation of The World still requires every continental dispute to be resolved and the final settlement ratified.</t>
         </is>
       </c>
@@ -24636,20 +24636,20 @@
       </c>
       <c r="C14" s="47" t="inlineStr">
         <is>
-          <t>A murder shakes the succession of an eligible government and opens an investigation into a hidden movement. Higher intensity gives it more reach and cohesion, and later discoveries may reveal threats beyond the first killing.</t>
+          <t xml:space="preserve">Begins the fictional Assassin Network crisis in an eligible government. The host suffers an opening succession shock and begins investigating a movement whose reach and cohesion grow with the selected intensity. Later discoveries may reveal threats beyond the original murder, while uninvolved countries retain their existing leadership.</t>
         </is>
       </c>
       <c r="D14" s="47" t="inlineStr">
         <is>
-          <t>Hidden Network</t>
+          <t xml:space="preserve">Clandestine network</t>
         </is>
       </c>
       <c r="E14" s="47" t="inlineStr">
         <is>
-          <t>§RStarts Assassin Network immediately.§! Low intensity opens a Murder Cult investigation with low reach and a small foreign network. No Assassin State exists at launch.
+          <t xml:space="preserve">§RStarts Assassin Network immediately.§! Low intensity opens a Murder Cult investigation with low reach and a small foreign network. No Assassin State exists at launch.
 §RStarts Assassin Network immediately.§! Medium intensity opens a mature international network and a stronger investigation. The host can still prevent the Assassin State split.
-§RStarts Assassin Network immediately.§! High intensity opens the Assassin State war and a strong foreign network.
-§RStarts Assassin Network immediately.§! Maximum intensity opens Evolution IV, the Assassin State war, and foreign operations. World of Anarchy still needs its usual end conditions.</t>
+§RStarts Assassin Network immediately.§! High intensity opens the Assassin State war and a strong foreign network through the normal country transaction.
+§RStarts Assassin Network immediately.§! Maximum intensity opens Evolution IV, the Assassin State war, and foreign derivative operations. World of Anarchy still requires its normal terminal conditions.</t>
         </is>
       </c>
       <c r="F14" s="70" t="inlineStr">

</xml_diff>

<commit_message>
Remove Fracture Cascade events and scenario while preserving civil wars
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -1775,7 +1775,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Manual_Scenarios" displayName="Manual_Scenarios" ref="A1:F17" headerRowCount="1" totalsRowShown="0" headerRowDxfId="43" headerRowBorderDxfId="42" tableBorderDxfId="41" totalsRowBorderDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Manual_Scenarios" displayName="Manual_Scenarios" ref="A1:F16" headerRowCount="1" totalsRowShown="0" headerRowDxfId="43" headerRowBorderDxfId="42" tableBorderDxfId="41" totalsRowBorderDxfId="40">
   <sortState ref="A2:F16">
     <sortCondition ref="A2:A16"/>
   </sortState>
@@ -3261,11 +3261,7 @@
           <t>Arms routes and foreign sponsors are carrying the crisis across borders. Civilian relief and armed support demand separate choices. The fighting sides are reorganizing their supplies, defenses and mobile columns. In a few units, night gatherings, sworn oaths and repeated signs have appeared that no one outside their ranks can explain.</t>
         </is>
       </c>
-      <c r="F22" s="37" t="inlineStr">
-        <is>
-          <t>Countries are moving from stability into exposure, fracture, and open crisis as divided commands and regional movements test weakened governments. Victory, reform, and negotiated terms can still restore public authority.</t>
-        </is>
-      </c>
+      <c r="F22" s="37" t="n"/>
       <c r="G22" s="38" t="n"/>
       <c r="H22" s="39" t="n"/>
       <c r="I22" s="40" t="n"/>
@@ -24155,7 +24151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.5703125" customWidth="1" min="1" max="1"/>
@@ -24732,45 +24728,6 @@
         </is>
       </c>
       <c r="F16" s="70" t="inlineStr">
-        <is>
-          <t>Needs Testing</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="46" t="inlineStr">
-        <is>
-          <t>SCN-018</t>
-        </is>
-      </c>
-      <c r="B17" s="47" t="inlineStr">
-        <is>
-          <t>The Fracture Cascade</t>
-        </is>
-      </c>
-      <c r="C17" s="47" t="inlineStr">
-        <is>
-          <t>Launch The Fracture Cascade against the selected share of eligible countries. The scenario creates internal wars without ending the world.
-Political Fracture: Prioritizes ideological uprisings, rival legal governments, coalition breakdowns, constitutional disputes, and seizures of central authority.
-Independence Cascade: Prioritizes established independence movements, regional secessions, recognition disputes, and wars of separation.
-Command Collapse: Prioritizes command schisms, military districts, arsenal seizures, officer disloyalty, and military seizures of central authority.
-Universal Fragmentation: Combines political, legal, military, regional, independence, and successor-state crises wherever each form can sustain a conflict.</t>
-        </is>
-      </c>
-      <c r="D17" s="47" t="inlineStr">
-        <is>
-          <t>Political Fracture, Independence Cascade, Command Collapse, Universal Fragmentation</t>
-        </is>
-      </c>
-      <c r="E17" s="47" t="inlineStr">
-        <is>
-          <t>Low: Roughly ten percent of eligible countries face limited uprisings with smaller territorial and military commitments.
-Medium: Roughly a quarter of eligible countries face stronger uprisings, established independence movements, and selected multi-front wars.
-High: Roughly half of eligible countries face frequent multi-front wars, stronger foreign pressure, and some crises within young successor states.
-Maximum: Every eligible country faces its strongest sustainable fracture. Countries outside ordinary human politics remain unaffected, and the scenario does not end the world.</t>
-        </is>
-      </c>
-      <c r="F17" s="70" t="inlineStr">
         <is>
           <t>Needs Testing</t>
         </is>
@@ -24798,7 +24755,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Unavailable,Needs Testing,Playable,To Be Reworked,Partially Available"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Restore Final Silence catalog scenario
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -1775,9 +1775,9 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Manual_Scenarios" displayName="Manual_Scenarios" ref="A1:F16" headerRowCount="1" totalsRowShown="0" headerRowDxfId="43" headerRowBorderDxfId="42" tableBorderDxfId="41" totalsRowBorderDxfId="40">
-  <sortState ref="A2:F16">
-    <sortCondition ref="A2:A16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Manual_Scenarios" displayName="Manual_Scenarios" ref="A1:F17" headerRowCount="1" totalsRowShown="0" headerRowDxfId="43" headerRowBorderDxfId="42" tableBorderDxfId="41" totalsRowBorderDxfId="40">
+  <sortState ref="A2:F17">
+    <sortCondition ref="A2:A17"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" name="Scenario ID" dataDxfId="39"/>
@@ -2222,7 +2222,10 @@
       <c r="H4" s="39" t="n"/>
       <c r="I4" s="87" t="inlineStr">
         <is>
-          <t>The Holy Realm completes its last rite and launches the Final Silence strikes. The last sanctuaries are destroyed, governments collapse, and the Awakened One leaves the Empty Seat to guard what survives.</t>
+          <t xml:space="preserve">Final Silence
+The Holy Realm's final rite ends in a nuclear catastrophe. Fallout follows the strike, destroying governments and leaving survivors to seek shelter.
+Fallout
+The Realm's final order has called in Fallout. The Empty Seat remains above the mountains as the last calamity overtakes the world.</t>
         </is>
       </c>
       <c r="J4" s="65" t="inlineStr">
@@ -24151,7 +24154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="11.5703125" customWidth="1" min="1" max="1"/>
@@ -24733,8 +24736,41 @@
         </is>
       </c>
     </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="47" t="inlineStr">
+        <is>
+          <t>SCN-004</t>
+        </is>
+      </c>
+      <c r="B17" s="47" t="inlineStr">
+        <is>
+          <t>Final Silence</t>
+        </is>
+      </c>
+      <c r="C17" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Starts the Final Silence world-end sequence from the current country with the nuclear variant. The launcher becomes the surviving Realm-side authority while every other valid state is struck in waves, suffers fallout, records deaths, and degrades toward wasteland.
+Starts the Final Silence world-end sequence from the current country with the thermonuclear variant. The launcher becomes the surviving Realm-side authority while every other valid state is struck in waves, suffers stronger fallout, records heavier deaths, and degrades toward wasteland.</t>
+        </is>
+      </c>
+      <c r="D17" s="47" t="inlineStr">
+        <is>
+          <t>Nuclear, Thermonuclear</t>
+        </is>
+      </c>
+      <c r="E17" s="47" t="inlineStr">
+        <is>
+          <t>Intensity does not change the sequence. The first wave strikes immediately, followed by waves across Asia and the Middle East, Europe and Africa, the Americas, then Oceania and the remaining regions at the existing wave interval. The sequence ends at 100% global air contamination. Nuclear payloads remove 75% of non-Realm civilian population; thermonuclear payloads remove 95%. The report opens after one day.</t>
+        </is>
+      </c>
+      <c r="F17" s="70" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F16">
+  <conditionalFormatting sqref="F2:F17">
     <cfRule type="expression" priority="1" dxfId="5" stopIfTrue="1">
       <formula>$F2="Partially Available"</formula>
     </cfRule>
@@ -24755,7 +24791,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Unavailable,Needs Testing,Playable,To Be Reworked,Partially Available"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Align the Event 38 catalog row with the in-game Event Details text
The Malta Crusaders Details cell now mirrors the shipped event details localisation, and the World-End Scenario cell is cleared because no terminal branch is implemented yet.
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -2222,7 +2222,7 @@
       <c r="H4" s="39" t="n"/>
       <c r="I4" s="87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Final Silence
+          <t>Final Silence
 The Holy Realm's final rite ends in a nuclear catastrophe. Fallout follows the strike, destroying governments and leaving survivors to seek shelter.
 Fallout
 The Realm's final order has called in Fallout. The Empty Seat remains above the mountains as the last calamity overtakes the world.</t>
@@ -2618,7 +2618,7 @@
       </c>
       <c r="D11" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Death reaches a second island and empties it slowly enough to resemble lost shipping or an abandoned harbor. The silence spreads from shore to shore while mainland governments remain uncertain of its cause.</t>
+          <t>Death reaches a second island and empties it slowly enough to resemble lost shipping or an abandoned harbor. The silence spreads from shore to shore while mainland governments remain uncertain of its cause.</t>
         </is>
       </c>
       <c r="E11" s="83" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="C12" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strangers keep meeting in the wrong places. Couriers vanish, equipment fails, and the same quiet methods turn up in distant incidents. Following the trail can expose the pattern, while practical precautions may blunt the next attack.</t>
+          <t>Strangers keep meeting in the wrong places. Couriers vanish, equipment fails, and the same quiet methods turn up in distant incidents. Following the trail can expose the pattern, while practical precautions may blunt the next attack.</t>
         </is>
       </c>
       <c r="D12" s="82" t="inlineStr">
@@ -2918,12 +2918,12 @@
       </c>
       <c r="G16" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Manifesto shapes regional politics. Governments invoke it when seeking aid, defending local charters, resisting threats, or seeking association. Small states must decide whether the commonwealth is a refuge, a useful partner, or an ambitious neighbor.</t>
+          <t>The Manifesto shapes regional politics. Governments invoke it when seeking aid, defending local charters, resisting threats, or seeking association. Small states must decide whether the commonwealth is a refuge, a useful partner, or an ambitious neighbor.</t>
         </is>
       </c>
       <c r="H16" s="86" t="inlineStr">
         <is>
-          <t xml:space="preserve">The world around the commonwealth is coming apart. Harbors, trains, fortifications, and refuge towns all need the same stores. Citizens and league members ask whether the gates will protect them, who must serve inside, and which neighbors will share the burden.</t>
+          <t>The world around the commonwealth is coming apart. Harbors, trains, fortifications, and refuge towns all need the same stores. Citizens and league members ask whether the gates will protect them, who must serve inside, and which neighbors will share the burden.</t>
         </is>
       </c>
       <c r="I16" s="40" t="n"/>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="D20" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">The soldiers from nowhere now have district staffs, proper rolls, and officers the government can actually hold responsible.</t>
+          <t>The soldiers from nowhere now have district staffs, proper rolls, and officers the government can actually hold responsible.</t>
         </is>
       </c>
       <c r="E20" s="83" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="B24" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOV Nuclear Bombs</t>
+          <t>SOV Nuclear Bombs</t>
         </is>
       </c>
       <c r="C24" s="30" t="inlineStr">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="C31" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">A man who remembers a later time appears in one country and proves it with a page of secrets and a forecast that comes true. The government chooses how he works with the state, and each piece of advice he gives must be carried out before its reward is paid. Foreign services copy his records, plant forgeries, offer him asylum and try to take him. The more the world acts on what he says, the less his memory of the future still describes it. Officials who depend on him begin to fight over him and the country that holds him may split, and as the order of the world loosens people from earlier centuries start to arrive.</t>
+          <t>A man who remembers a later time appears in one country and proves it with a page of secrets and a forecast that comes true. The government chooses how he works with the state, and each piece of advice he gives must be carried out before its reward is paid. Foreign services copy his records, plant forgeries, offer him asylum and try to take him. The more the world acts on what he says, the less his memory of the future still describes it. Officials who depend on him begin to fight over him and the country that holds him may split, and as the order of the world loosens people from earlier centuries start to arrive.</t>
         </is>
       </c>
       <c r="D31" s="82" t="inlineStr">
@@ -3794,12 +3794,12 @@
       </c>
       <c r="C33" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Missile programmes have spread across the world. Countries can build and harden launch sites, stock operational missiles, improve guidance, and secure the officers and codes that control them. Heavier arsenals, guidance failures, special warheads, rogue commands, and automatic retaliation can transform the crisis.</t>
+          <t>Missile programmes have spread across the world. Countries can build and harden launch sites, stock operational missiles, improve guidance, and secure the officers and codes that control them. Heavier arsenals, guidance failures, special warheads, rogue commands, and automatic retaliation can transform the crisis.</t>
         </is>
       </c>
       <c r="D33" s="35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Countries with working launch sites and enough industry can adopt a saturation doctrine for massed salvos. Saturation attacks can overwhelm defences, but they consume many missiles and strain readiness and command control.</t>
+          <t>Countries with working launch sites and enough industry can adopt a saturation doctrine for massed salvos. Saturation attacks can overwhelm defences, but they consume many missiles and strain readiness and command control.</t>
         </is>
       </c>
       <c r="E33" s="36" t="inlineStr">
@@ -3809,7 +3809,7 @@
       </c>
       <c r="F33" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Countries that already possess chemical, biological, nuclear, or thermonuclear weapons can adapt them for missile delivery. Each launch still requires an authorised warhead held in secure custody.</t>
+          <t>Countries that already possess chemical, biological, nuclear, or thermonuclear weapons can adapt them for missile delivery. Each launch still requires an authorised warhead held in secure custody.</t>
         </is>
       </c>
       <c r="G33" s="38" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="F34" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Global Acid Rain: The fronts merge into a worldwide layer that exposes every valid inhabited state and produces regional superstorms with nine-day forecasts.</t>
+          <t>Global Acid Rain: The fronts merge into a worldwide layer that exposes every valid inhabited state and produces regional superstorms with nine-day forecasts.</t>
         </is>
       </c>
       <c r="G34" s="38" t="n"/>
@@ -4104,17 +4104,13 @@
       </c>
       <c r="C39" s="30" t="inlineStr">
         <is>
-          <t>Malta becomes independent, raises knightly armies, claims Mediterranean territory, and wages a new crusade. Later stages can place the Pope in Rome at the head of a Kingdom of God.</t>
+          <t>The Order of Saint John rises as a crusader state. It holds Malta, Jerusalem and a chain of harbours and fortified towns in between, and the governments it took them from are at war with it from the first day. Knights in plate march beside infantry in field grey, the military orders quarrel over who commands them, and the Pope and the Catholic world watch the Grand Master. A defeat in the Holy Land leads to a second crusade to win it back, and a world at higher Chaos draws more orders, more territory and more relics into the war.</t>
         </is>
       </c>
       <c r="D39" s="35" t="n"/>
       <c r="E39" s="36" t="n"/>
       <c r="F39" s="37" t="n"/>
-      <c r="G39" s="85" t="inlineStr">
-        <is>
-          <t>A dedicated crusader route opens. Failure leads to an eleventh crusade, while success expands the conquests, adopts The Holy See identity, installs the Pope as leader, and makes Rome the holy capital of a Kingdom of God.</t>
-        </is>
-      </c>
+      <c r="G39" s="85" t="n"/>
       <c r="H39" s="39" t="n"/>
       <c r="I39" s="40" t="n"/>
       <c r="J39" s="65" t="inlineStr">
@@ -4758,7 +4754,7 @@
       </c>
       <c r="B55" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Random Tech</t>
+          <t>Random Tech</t>
         </is>
       </c>
       <c r="C55" s="30" t="inlineStr">
@@ -4914,7 +4910,7 @@
       </c>
       <c r="B59" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Free Civs</t>
+          <t>Free Civs</t>
         </is>
       </c>
       <c r="C59" s="30" t="inlineStr">
@@ -5031,7 +5027,7 @@
       </c>
       <c r="B62" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mils into Civs</t>
+          <t>Mils into Civs</t>
         </is>
       </c>
       <c r="C62" s="30" t="inlineStr">
@@ -5187,7 +5183,7 @@
       </c>
       <c r="B66" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Random Trait</t>
+          <t>Random Trait</t>
         </is>
       </c>
       <c r="C66" s="30" t="inlineStr">
@@ -5222,7 +5218,7 @@
       </c>
       <c r="B67" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">CIC</t>
+          <t>CIC</t>
         </is>
       </c>
       <c r="C67" s="30" t="inlineStr">
@@ -5488,7 +5484,7 @@
       </c>
       <c r="B75" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Japan California</t>
+          <t>Japan California</t>
         </is>
       </c>
       <c r="C75" s="30" t="inlineStr">
@@ -5768,7 +5764,7 @@
       </c>
       <c r="B83" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Law Upgrade</t>
+          <t>Law Upgrade</t>
         </is>
       </c>
       <c r="C83" s="30" t="inlineStr">
@@ -6157,7 +6153,7 @@
       </c>
       <c r="B94" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Portugal Galicia</t>
+          <t>Portugal Galicia</t>
         </is>
       </c>
       <c r="C94" s="30" t="inlineStr">
@@ -6262,7 +6258,7 @@
       </c>
       <c r="B97" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Divisions Lock</t>
+          <t>Divisions Lock</t>
         </is>
       </c>
       <c r="C97" s="30" t="inlineStr">
@@ -21176,7 +21172,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sudden wars and armed conflicts break out between countries, turning local disputes, opportunistic attacks, and border shocks into a wider chain of fighting.</t>
+          <t>Sudden wars and armed conflicts break out between countries, turning local disputes, opportunistic attacks, and border shocks into a wider chain of fighting.</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -21247,12 +21243,12 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diplomatic Panic</t>
+          <t>Diplomatic Panic</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diplomatic crises spread through public quarrels, collapsing relations, hurried guarantees, and minor states pressed to choose among nearby blocs.</t>
+          <t>Diplomatic crises spread through public quarrels, collapsing relations, hurried guarantees, and minor states pressed to choose among nearby blocs.</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -21366,7 +21362,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Formables gather negotiated restoration and union projects. Africa Is One builds a protection-first Charter League through aid, guarantees, liberation recognition, consent, constitutional routes, and rival settlements. The Formables cluster remains repeatable; Africa Is One is its Severe Event 12 member, a tier-4 Minor Fire-Once entry with entry event chaosx.nr12.1.</t>
+          <t>Formables gather negotiated restoration and union projects. Africa Is One builds a protection-first Charter League through aid, guarantees, liberation recognition, consent, constitutional routes, and rival settlements. The Formables cluster remains repeatable; Africa Is One is its Severe Event 12 member, a tier-4 Minor Fire-Once entry with entry event chaosx.nr12.1.</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -21632,7 +21628,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Severe outbreaks establish persistent conditions in affected states. Each disease follows its own transmission routes and demands material, military, and time investment to contain it.</t>
+          <t>Severe outbreaks establish persistent conditions in affected states. Each disease follows its own transmission routes and demands material, military, and time investment to contain it.</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -22430,7 +22426,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diplomatic Panic</t>
+          <t>Diplomatic Panic</t>
         </is>
       </c>
       <c r="C16" s="5" t="n">
@@ -22457,7 +22453,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diplomatic Panic</t>
+          <t>Diplomatic Panic</t>
         </is>
       </c>
       <c r="C17" s="5" t="n">
@@ -22484,7 +22480,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diplomatic Panic</t>
+          <t>Diplomatic Panic</t>
         </is>
       </c>
       <c r="C18" s="5" t="n">
@@ -22511,7 +22507,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diplomatic Panic</t>
+          <t>Diplomatic Panic</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
@@ -22677,7 +22673,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mils into Civs</t>
+          <t>Mils into Civs</t>
         </is>
       </c>
       <c r="F24" s="54" t="inlineStr">
@@ -23162,7 +23158,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Free Civs</t>
+          <t>Free Civs</t>
         </is>
       </c>
       <c r="F41" s="54" t="inlineStr">
@@ -23274,7 +23270,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Random Tech</t>
+          <t>Random Tech</t>
         </is>
       </c>
       <c r="F45" s="54" t="inlineStr">
@@ -23301,7 +23297,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Random Trait</t>
+          <t>Random Trait</t>
         </is>
       </c>
       <c r="F46" s="54" t="inlineStr">
@@ -24306,7 +24302,7 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pact: Turns eligible non-player minor countries into dispersed Fury actors and organizes them into the Fury Pact. Higher intensity spreads more Fury states across the world and grants stronger evolved openings.
+          <t>Pact: Turns eligible non-player minor countries into dispersed Fury actors and organizes them into the Fury Pact. Higher intensity spreads more Fury states across the world and grants stronger evolved openings.
 Hostile: Turns eligible non-player minor countries into dispersed hostile Fury actors that immediately pursue neighboring wars. Higher intensity spreads more Fury states across the world and escalates their opening pressure.</t>
         </is>
       </c>
@@ -24406,7 +24402,7 @@
       </c>
       <c r="C8" s="52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sovereign Scatter: Every viable movement is attempted. Each release keeps a protected former-host remnant and unique anchor. States remain outside pre-formed leagues and retain no release-created faction ties. Intensity changes territory, forces, institutions, and pressure.
+          <t>Sovereign Scatter: Every viable movement is attempted. Each release keeps a protected former-host remnant and unique anchor. States remain outside pre-formed leagues and retain no release-created faction ties. Intensity changes territory, forces, institutions, and pressure.
 Open Congress: Every viable movement is attempted under protected hosts and unique anchors. New states join an informal congress network. Higher intensity strengthens its charter and shared reserve.
 Separation Wars: Every viable movement is attempted. A country that can lawfully confront its surviving former host may open one separation war. Others receive a regional threat mission.
 Host Wars: Every viable movement is attempted. Each new country may face one bounded former-host conflict. Invalid declarations become regional threat missions. Host remnants and homelands are secured first.
@@ -24423,7 +24419,7 @@
       </c>
       <c r="E8" s="52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low: All viable candidates are still attempted. Each valid release receives only its anchor, fragile local defense, scarce stocks, weak institutions, low recognition, and severe opening instability.
+          <t>Low: All viable candidates are still attempted. Each valid release receives only its anchor, fragile local defense, scarce stocks, weak institutions, low recognition, and severe opening instability.
 Medium: All viable candidates are still attempted. Valid releases receive compact territory, viable militia and border formations, baseline institutions, and ordinary route access.
 High: All viable candidates are still attempted. Valid releases receive extended territory where collisions permit, armed forces, stronger depots and officers, firmer institutions, faster league development, and accelerated ambitions.
 Maximum: All viable candidates are still attempted. Valid releases receive the strongest non-overlapping territory and forces, rare support where their researched route permits it, high-chaos access, early formable discovery, and aggressive AI pressure.</t>
@@ -24526,7 +24522,7 @@
       </c>
       <c r="C11" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Africa Is One: Forms a strong Africa, opens the Charter League, regional authority, Authority Atlas, sponsor, proof-ledger, and post-unification systems, then opens the continental unification war office.
+          <t>Africa Is One: Forms a strong Africa, opens the Charter League, regional authority, Authority Atlas, sponsor, proof-ledger, and post-unification systems, then opens the continental unification war office.
 World Is One: Forms Africa and prepares the World Is One final campaign. Rival continental powers become eligible for treaties, containment, or war, while the proclamation of The World still requires every continental dispute to be resolved and the final settlement ratified.</t>
         </is>
       </c>
@@ -24635,17 +24631,17 @@
       </c>
       <c r="C14" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Begins the fictional Assassin Network crisis in an eligible government. The host suffers an opening succession shock and begins investigating a movement whose reach and cohesion grow with the selected intensity. Later discoveries may reveal threats beyond the original murder, while uninvolved countries retain their existing leadership.</t>
+          <t>Begins the fictional Assassin Network crisis in an eligible government. The host suffers an opening succession shock and begins investigating a movement whose reach and cohesion grow with the selected intensity. Later discoveries may reveal threats beyond the original murder, while uninvolved countries retain their existing leadership.</t>
         </is>
       </c>
       <c r="D14" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Clandestine network</t>
+          <t>Clandestine network</t>
         </is>
       </c>
       <c r="E14" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">§RStarts Assassin Network immediately.§! Low intensity opens a Murder Cult investigation with low reach and a small foreign network. No Assassin State exists at launch.
+          <t>§RStarts Assassin Network immediately.§! Low intensity opens a Murder Cult investigation with low reach and a small foreign network. No Assassin State exists at launch.
 §RStarts Assassin Network immediately.§! Medium intensity opens a mature international network and a stronger investigation. The host can still prevent the Assassin State split.
 §RStarts Assassin Network immediately.§! High intensity opens the Assassin State war and a strong foreign network through the normal country transaction.
 §RStarts Assassin Network immediately.§! Maximum intensity opens Evolution IV, the Assassin State war, and foreign derivative operations. World of Anarchy still requires its normal terminal conditions.</t>
@@ -24736,7 +24732,7 @@
         </is>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17">
       <c r="A17" s="47" t="inlineStr">
         <is>
           <t>SCN-004</t>
@@ -24749,7 +24745,7 @@
       </c>
       <c r="C17" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Starts the Final Silence world-end sequence from the current country with the nuclear variant. The launcher becomes the surviving Realm-side authority while every other valid state is struck in waves, suffers fallout, records deaths, and degrades toward wasteland.
+          <t>Starts the Final Silence world-end sequence from the current country with the nuclear variant. The launcher becomes the surviving Realm-side authority while every other valid state is struck in waves, suffers fallout, records deaths, and degrades toward wasteland.
 Starts the Final Silence world-end sequence from the current country with the thermonuclear variant. The launcher becomes the surviving Realm-side authority while every other valid state is struck in waves, suffers stronger fallout, records heavier deaths, and degrades toward wasteland.</t>
         </is>
       </c>
@@ -24760,7 +24756,7 @@
       </c>
       <c r="E17" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Intensity does not change the four-wave sequence. The first wave begins immediately in Asia and the Middle East; the remaining waves follow at the existing interval through Europe and Africa, the Americas, and Oceania and the remaining regions. The sequence ends at 100% global air contamination. Nuclear payloads remove 75% of non-Realm civilian population; thermonuclear payloads remove 95%. The report opens after one day.</t>
+          <t>Intensity does not change the four-wave sequence. The first wave begins immediately in Asia and the Middle East; the remaining waves follow at the existing interval through Europe and Africa, the Americas, and Oceania and the remaining regions. The sequence ends at 100% global air contamination. Nuclear payloads remove 75% of non-Realm civilian population; thermonuclear payloads remove 95%. The report opens after one day.</t>
         </is>
       </c>
       <c r="F17" s="70" t="inlineStr">

</xml_diff>

<commit_message>
Import event planning packages and align catalog identities
Import and reconcile the eight supplied event packages. Adopt their catalog
identities, preserve displaced concepts, and update dependent references.

Specify the worldwide free Lootboxes opening and Fuel Crisis Severe
membership in Various Anomalies. Preserve runtime availability boundaries.
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -1760,7 +1760,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Cluster_Memberships" displayName="Cluster_Memberships" ref="A1:G77" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Cluster_Memberships" displayName="Cluster_Memberships" ref="A1:G78" headerRowCount="1">
   <tableColumns count="7">
     <tableColumn id="1" name="Cluster ID"/>
     <tableColumn id="2" name="Cluster Name"/>
@@ -6512,12 +6512,12 @@
       </c>
       <c r="B105" s="30" t="inlineStr">
         <is>
-          <t>Stability or War support</t>
+          <t>Rule</t>
         </is>
       </c>
       <c r="C105" s="30" t="inlineStr">
         <is>
-          <t>Each country weighs stability against war support, gaining one while sacrificing the other.</t>
+          <t>A random rule becomes active and changes the campaign.</t>
         </is>
       </c>
       <c r="D105" s="35" t="n"/>
@@ -6541,12 +6541,12 @@
       </c>
       <c r="B106" s="30" t="inlineStr">
         <is>
-          <t>Anti-player ideology</t>
+          <t>Random Idea</t>
         </is>
       </c>
       <c r="C106" s="30" t="inlineStr">
         <is>
-          <t>A player's ideology faces temporary decline and public discontent. Protest movements are weaker when support is high, while a collapse below one percent can trigger regime change or civil war.</t>
+          <t>A national spirit appears in every country, bringing an unpredictable change to national life.</t>
         </is>
       </c>
       <c r="D106" s="35" t="n"/>
@@ -6570,12 +6570,12 @@
       </c>
       <c r="B107" s="30" t="inlineStr">
         <is>
-          <t>Paranoia</t>
+          <t>Resistance</t>
         </is>
       </c>
       <c r="C107" s="30" t="inlineStr">
         <is>
-          <t>A paranoia crisis spreads through a country in a manner similar to the Soviet Union crisis.</t>
+          <t>Occupied states erupt in resistance across major countries and the player.</t>
         </is>
       </c>
       <c r="D107" s="35" t="n"/>
@@ -6599,12 +6599,12 @@
       </c>
       <c r="B108" s="30" t="inlineStr">
         <is>
-          <t>Rule</t>
+          <t>Lootboxes</t>
         </is>
       </c>
       <c r="C108" s="30" t="inlineStr">
         <is>
-          <t>A random rule becomes active and changes the campaign.</t>
+          <t>Mysterious chests appear in every country. Each government receives its first chest as a gift, and a permanent market offers further boxes with unpredictable prizes.</t>
         </is>
       </c>
       <c r="D108" s="35" t="n"/>
@@ -6628,12 +6628,12 @@
       </c>
       <c r="B109" s="30" t="inlineStr">
         <is>
-          <t>Fury</t>
+          <t>Wrestling Tournament</t>
         </is>
       </c>
       <c r="C109" s="30" t="inlineStr">
         <is>
-          <t>A small non-island country launches an expansionist campaign.</t>
+          <t>A wrestling tournament rewards the champion after countries train their chosen contender.</t>
         </is>
       </c>
       <c r="D109" s="35" t="n"/>
@@ -6657,12 +6657,12 @@
       </c>
       <c r="B110" s="30" t="inlineStr">
         <is>
-          <t>Custom laws</t>
+          <t>Fuel Crisis</t>
         </is>
       </c>
       <c r="C110" s="30" t="inlineStr">
         <is>
-          <t>A new national spirit appears in every country.</t>
+          <t>A worldwide fuel crisis leaves every country with no stored fuel.</t>
         </is>
       </c>
       <c r="D110" s="35" t="n"/>
@@ -6673,7 +6673,11 @@
       <c r="I110" s="40" t="n"/>
       <c r="J110" s="43" t="n"/>
       <c r="K110" s="54" t="n"/>
-      <c r="L110" s="54" t="n"/>
+      <c r="L110" s="54" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="M110" s="73" t="inlineStr">
         <is>
           <t>Unavailable</t>
@@ -6686,12 +6690,12 @@
       </c>
       <c r="B111" s="30" t="inlineStr">
         <is>
-          <t>Random idea</t>
+          <t>IMRO</t>
         </is>
       </c>
       <c r="C111" s="30" t="inlineStr">
         <is>
-          <t>Occupied states erupt in resistance across major countries and the player.</t>
+          <t>A Macedonian uprising turns the slogan Freedom or Death into a national crisis.</t>
         </is>
       </c>
       <c r="D111" s="35" t="n"/>
@@ -6715,12 +6719,12 @@
       </c>
       <c r="B112" s="30" t="inlineStr">
         <is>
-          <t>Resistance</t>
+          <t>This is SPARTA!!!</t>
         </is>
       </c>
       <c r="C112" s="30" t="inlineStr">
         <is>
-          <t>A chest market introduces common, rare, and epic prizes to a country's political life.</t>
+          <t>Spartan warriors rise in Greece.</t>
         </is>
       </c>
       <c r="D112" s="35" t="n"/>
@@ -6744,12 +6748,12 @@
       </c>
       <c r="B113" s="30" t="inlineStr">
         <is>
-          <t>Lootboxes</t>
+          <t>Rise of Cossacks</t>
         </is>
       </c>
       <c r="C113" s="30" t="inlineStr">
         <is>
-          <t>A national wrestling tournament turns one contender into a public hero.</t>
+          <t>Cossacks rise from a random East Slavic state and expand across East Slavia.</t>
         </is>
       </c>
       <c r="D113" s="35" t="n"/>
@@ -6773,12 +6777,12 @@
       </c>
       <c r="B114" s="30" t="inlineStr">
         <is>
-          <t>Wrestling Tournament</t>
+          <t>The Partition</t>
         </is>
       </c>
       <c r="C114" s="30" t="inlineStr">
         <is>
-          <t>A wrestling tournament rewards the champion after countries train their chosen contender.</t>
+          <t>Several neighbors claim a random country and divide its territory or fight for it.</t>
         </is>
       </c>
       <c r="D114" s="35" t="n"/>
@@ -6802,12 +6806,12 @@
       </c>
       <c r="B115" s="30" t="inlineStr">
         <is>
-          <t>Fuel crisis</t>
+          <t>Demilitarization</t>
         </is>
       </c>
       <c r="C115" s="30" t="inlineStr">
         <is>
-          <t>A worldwide fuel crisis leaves every country with no stored fuel.</t>
+          <t>Countries at peace demilitarize every state except their capital until war allows remilitarization.</t>
         </is>
       </c>
       <c r="D115" s="35" t="n"/>
@@ -6831,12 +6835,12 @@
       </c>
       <c r="B116" s="30" t="inlineStr">
         <is>
-          <t>IMRO</t>
+          <t>Heroic Crusade</t>
         </is>
       </c>
       <c r="C116" s="30" t="inlineStr">
         <is>
-          <t>A Macedonian uprising turns the slogan Freedom or Death into a national crisis.</t>
+          <t>A religious faction forms with the goal of destroying rival religions.</t>
         </is>
       </c>
       <c r="D116" s="35" t="n"/>
@@ -6860,12 +6864,12 @@
       </c>
       <c r="B117" s="30" t="inlineStr">
         <is>
-          <t>This is SPARTA!!!</t>
+          <t>Warlords</t>
         </is>
       </c>
       <c r="C117" s="30" t="inlineStr">
         <is>
-          <t>Spartan warriors rise in Greece.</t>
+          <t>Regional commanders break away from weakened governments, building rival states that struggle for territory, loyalty, and survival.</t>
         </is>
       </c>
       <c r="D117" s="35" t="n"/>
@@ -6889,12 +6893,12 @@
       </c>
       <c r="B118" s="30" t="inlineStr">
         <is>
-          <t>5-Way Civil War</t>
+          <t>Autonomy</t>
         </is>
       </c>
       <c r="C118" s="30" t="inlineStr">
         <is>
-          <t>A major country or the player faces five rival camps in a civil war. Stability and ideology support shape the opening balance, while alliances can postpone the final duel.</t>
+          <t>Every subject receives autonomy points.</t>
         </is>
       </c>
       <c r="D118" s="35" t="n"/>
@@ -6918,12 +6922,12 @@
       </c>
       <c r="B119" s="30" t="inlineStr">
         <is>
-          <t>Plague of locust</t>
+          <t>Shaman</t>
         </is>
       </c>
       <c r="C119" s="30" t="inlineStr">
         <is>
-          <t>A plague of locusts travels across the world and brings famine to affected regions.</t>
+          <t>A regional shaman offers aid to the major country that controls the surrounding area.</t>
         </is>
       </c>
       <c r="D119" s="35" t="n"/>
@@ -6947,12 +6951,12 @@
       </c>
       <c r="B120" s="30" t="inlineStr">
         <is>
-          <t>Random New Alliance</t>
+          <t>Mistresses</t>
         </is>
       </c>
       <c r="C120" s="30" t="inlineStr">
         <is>
-          <t>A new regional alliance forms in a random part of the world.</t>
+          <t>Tomorrow's Girls brings alien companions into national politics, and a leader can gain manpower through their influence.</t>
         </is>
       </c>
       <c r="D120" s="35" t="n"/>
@@ -6976,12 +6980,12 @@
       </c>
       <c r="B121" s="30" t="inlineStr">
         <is>
-          <t>Massive Volcano Eruption</t>
+          <t>Widespread Mutiny</t>
         </is>
       </c>
       <c r="C121" s="30" t="inlineStr">
         <is>
-          <t>A massive volcanic eruption turns the states around a random volcanic region into wasteland.</t>
+          <t>Countries with low war support face army mutinies as units turn against their commands.</t>
         </is>
       </c>
       <c r="D121" s="35" t="n"/>
@@ -7005,12 +7009,12 @@
       </c>
       <c r="B122" s="30" t="inlineStr">
         <is>
-          <t>The Pact</t>
+          <t>Investment</t>
         </is>
       </c>
       <c r="C122" s="30" t="inlineStr">
         <is>
-          <t>The strongest country in a random ideology proposes a pact in which every member guarantees the others.</t>
+          <t>A government invests in military, civilian, naval, or special industry.</t>
         </is>
       </c>
       <c r="D122" s="35" t="n"/>
@@ -7034,12 +7038,12 @@
       </c>
       <c r="B123" s="30" t="inlineStr">
         <is>
-          <t>Rise of Cossacks</t>
+          <t>Gandhi</t>
         </is>
       </c>
       <c r="C123" s="30" t="inlineStr">
         <is>
-          <t>Cossacks rise from a random East Slavic state and expand across East Slavia.</t>
+          <t>Countries holding non-core states face independence movements shaped by Gandhi's principles of nonviolence, noncooperation, truth, and honesty. Denial removes the value of occupation while unrest spreads, with fascist governments affected differently.</t>
         </is>
       </c>
       <c r="D123" s="35" t="n"/>
@@ -7059,16 +7063,16 @@
     </row>
     <row r="124" ht="22.5" customHeight="1">
       <c r="A124" s="34" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B124" s="30" t="inlineStr">
         <is>
-          <t>The Partition</t>
+          <t>Non-Aggressions</t>
         </is>
       </c>
       <c r="C124" s="30" t="inlineStr">
         <is>
-          <t>Several neighbors claim a random country and divide its territory or fight for it.</t>
+          <t>Two random countries sign a non-aggression pact.</t>
         </is>
       </c>
       <c r="D124" s="35" t="n"/>
@@ -7088,16 +7092,16 @@
     </row>
     <row r="125" ht="22.5" customHeight="1">
       <c r="A125" s="34" t="n">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="B125" s="30" t="inlineStr">
         <is>
-          <t>Demilitarization</t>
+          <t>Duchies</t>
         </is>
       </c>
       <c r="C125" s="30" t="inlineStr">
         <is>
-          <t>Countries at peace demilitarize every state except their capital until war allows remilitarization.</t>
+          <t>Countries face a sudden surplus of military equipment.</t>
         </is>
       </c>
       <c r="D125" s="35" t="n"/>
@@ -7117,16 +7121,16 @@
     </row>
     <row r="126" ht="22.5" customHeight="1">
       <c r="A126" s="34" t="n">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="B126" s="30" t="inlineStr">
         <is>
-          <t>Non-Aggressions</t>
+          <t>Equipment choice</t>
         </is>
       </c>
       <c r="C126" s="30" t="inlineStr">
         <is>
-          <t>Two random countries sign a non-aggression pact.</t>
+          <t>Every country receives a choice of large equipment grants.</t>
         </is>
       </c>
       <c r="D126" s="35" t="n"/>
@@ -7146,16 +7150,16 @@
     </row>
     <row r="127" ht="22.5" customHeight="1">
       <c r="A127" s="34" t="n">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="B127" s="30" t="inlineStr">
         <is>
-          <t>Heroic Crusade</t>
+          <t>Sun moves away</t>
         </is>
       </c>
       <c r="C127" s="30" t="inlineStr">
         <is>
-          <t>A religious faction forms with the goal of destroying rival religions.</t>
+          <t>A research surge focuses each country on one field.</t>
         </is>
       </c>
       <c r="D127" s="35" t="n"/>
@@ -7175,16 +7179,16 @@
     </row>
     <row r="128" ht="22.5" customHeight="1">
       <c r="A128" s="34" t="n">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="B128" s="30" t="inlineStr">
         <is>
-          <t>Warlords</t>
+          <t>Research Investment</t>
         </is>
       </c>
       <c r="C128" s="30" t="inlineStr">
         <is>
-          <t>Subject governments demand greater autonomy.</t>
+          <t>Every country receives a choice of research investment in one category.</t>
         </is>
       </c>
       <c r="D128" s="35" t="n"/>
@@ -7204,16 +7208,16 @@
     </row>
     <row r="129" ht="22.5" customHeight="1">
       <c r="A129" s="34" t="n">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="B129" s="30" t="inlineStr">
         <is>
-          <t>Autonomy</t>
+          <t>The Kingdom of the Mountains</t>
         </is>
       </c>
       <c r="C129" s="30" t="inlineStr">
         <is>
-          <t>Every subject receives autonomy points.</t>
+          <t>A mountain and hill country forms the Mountain Republic and claims every matching state.</t>
         </is>
       </c>
       <c r="D129" s="35" t="n"/>
@@ -7233,16 +7237,16 @@
     </row>
     <row r="130" ht="22.5" customHeight="1">
       <c r="A130" s="34" t="n">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="B130" s="30" t="inlineStr">
         <is>
-          <t>Shaman</t>
+          <t>Mysterious creature</t>
         </is>
       </c>
       <c r="C130" s="30" t="inlineStr">
         <is>
-          <t>A regional shaman offers aid to the major country that controls the surrounding area.</t>
+          <t>A creature feeds on crops and people in a random major country or the player, spreading fear until it is hunted.</t>
         </is>
       </c>
       <c r="D130" s="35" t="n"/>
@@ -7262,16 +7266,16 @@
     </row>
     <row r="131" ht="22.5" customHeight="1">
       <c r="A131" s="34" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="B131" s="30" t="inlineStr">
         <is>
-          <t>Mistresses</t>
+          <t>Dracula</t>
         </is>
       </c>
       <c r="C131" s="30" t="inlineStr">
         <is>
-          <t>Tomorrow's Girls brings alien companions into national politics, and a leader can gain manpower through their influence.</t>
+          <t>Dracula terrorizes Transylvania and can found the Vampire Kingdom, which attacks its former controller and England before threatening the world. The one-battalion “Count Dracula” unit decides the kingdom's fate, and neighbors receive the “Fear of Dracula” national spirit until they confront it.</t>
         </is>
       </c>
       <c r="D131" s="35" t="n"/>
@@ -7291,16 +7295,16 @@
     </row>
     <row r="132" ht="22.5" customHeight="1">
       <c r="A132" s="34" t="n">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="B132" s="30" t="inlineStr">
         <is>
-          <t>Widespread Mutiny</t>
+          <t>Mass suicides</t>
         </is>
       </c>
       <c r="C132" s="30" t="inlineStr">
         <is>
-          <t>Countries with low war support face army mutinies as units turn against their commands.</t>
+          <t>Whispers drive mass suicides in a random major country or the player. As deaths spread, generals and leaders can disappear until the country itself collapses.</t>
         </is>
       </c>
       <c r="D132" s="35" t="n"/>
@@ -7320,16 +7324,16 @@
     </row>
     <row r="133" ht="22.5" customHeight="1">
       <c r="A133" s="34" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="B133" s="30" t="inlineStr">
         <is>
-          <t>Investment</t>
+          <t>Partisans</t>
         </is>
       </c>
       <c r="C133" s="30" t="inlineStr">
         <is>
-          <t>A government invests in military, civilian, naval, or special industry.</t>
+          <t>A major country or player with strong ideological support faces partisan divisions, some of them armored, in proportion to its support.</t>
         </is>
       </c>
       <c r="D133" s="35" t="n"/>
@@ -7349,16 +7353,16 @@
     </row>
     <row r="134" ht="22.5" customHeight="1">
       <c r="A134" s="34" t="n">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="B134" s="30" t="inlineStr">
         <is>
-          <t>Gandhi</t>
+          <t>A Game</t>
         </is>
       </c>
       <c r="C134" s="30" t="inlineStr">
         <is>
-          <t>Countries holding non-core states face independence movements shaped by Gandhi's principles of nonviolence, noncooperation, truth, and honesty. Denial removes the value of occupation while unrest spreads, with fascist governments affected differently.</t>
+          <t>A rock-paper-scissors contest decides a territorial dispute. Victory transfers the state, while defeat costs part of the player's industry.</t>
         </is>
       </c>
       <c r="D134" s="35" t="n"/>
@@ -7378,16 +7382,16 @@
     </row>
     <row r="135" ht="22.5" customHeight="1">
       <c r="A135" s="34" t="n">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="B135" s="30" t="inlineStr">
         <is>
-          <t>Duchies</t>
+          <t>Freedom or Death</t>
         </is>
       </c>
       <c r="C135" s="30" t="inlineStr">
         <is>
-          <t>Countries face a sudden surplus of military equipment.</t>
+          <t>Subjects across the world declare independence and form the National Liberation Front. Their former masters can accept the separation or fight the simultaneous wars.</t>
         </is>
       </c>
       <c r="D135" s="35" t="n"/>
@@ -7407,16 +7411,16 @@
     </row>
     <row r="136" ht="22.5" customHeight="1">
       <c r="A136" s="34" t="n">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="B136" s="30" t="inlineStr">
         <is>
-          <t>Equipment choice</t>
+          <t>The Book</t>
         </is>
       </c>
       <c r="C136" s="30" t="inlineStr">
         <is>
-          <t>Every country receives a choice of large equipment grants.</t>
+          <t>Intelligence agencies expand their clandestine networks.</t>
         </is>
       </c>
       <c r="D136" s="35" t="n"/>
@@ -7436,16 +7440,16 @@
     </row>
     <row r="137" ht="22.5" customHeight="1">
       <c r="A137" s="34" t="n">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="B137" s="30" t="inlineStr">
         <is>
-          <t>Sun moves away</t>
+          <t>Add operative</t>
         </is>
       </c>
       <c r="C137" s="30" t="inlineStr">
         <is>
-          <t>A research surge focuses each country on one field.</t>
+          <t>Counterintelligence improves across the world.</t>
         </is>
       </c>
       <c r="D137" s="35" t="n"/>
@@ -7465,16 +7469,16 @@
     </row>
     <row r="138" ht="22.5" customHeight="1">
       <c r="A138" s="34" t="n">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="B138" s="30" t="inlineStr">
         <is>
-          <t>Research Investment</t>
+          <t>Counterintelligence</t>
         </is>
       </c>
       <c r="C138" s="30" t="inlineStr">
         <is>
-          <t>Every country receives a choice of research investment in one category.</t>
+          <t>Every country gains one point of counterintelligence.</t>
         </is>
       </c>
       <c r="D138" s="35" t="n"/>
@@ -7494,16 +7498,16 @@
     </row>
     <row r="139" ht="22.5" customHeight="1">
       <c r="A139" s="34" t="n">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="B139" s="30" t="inlineStr">
         <is>
-          <t>The Kingdom of the Mountains</t>
+          <t>Pacifism</t>
         </is>
       </c>
       <c r="C139" s="30" t="inlineStr">
         <is>
-          <t>A mountain and hill country forms the Mountain Republic and claims every matching state.</t>
+          <t>Pacifism rises again as a political force.</t>
         </is>
       </c>
       <c r="D139" s="35" t="n"/>
@@ -7523,16 +7527,16 @@
     </row>
     <row r="140" ht="22.5" customHeight="1">
       <c r="A140" s="34" t="n">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="B140" s="30" t="inlineStr">
         <is>
-          <t>Mysterious creature</t>
+          <t>Immigrations</t>
         </is>
       </c>
       <c r="C140" s="30" t="inlineStr">
         <is>
-          <t>A creature feeds on crops and people in a random major country or the player, spreading fear until it is hunted.</t>
+          <t>Retired and absorbed into the separate famine and migration mechanics through explicit adapters. Unavailable as a random event.</t>
         </is>
       </c>
       <c r="D140" s="35" t="n"/>
@@ -7552,16 +7556,16 @@
     </row>
     <row r="141" ht="22.5" customHeight="1">
       <c r="A141" s="34" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="B141" s="30" t="inlineStr">
         <is>
-          <t>Dracula</t>
+          <t>Secret Society Influence</t>
         </is>
       </c>
       <c r="C141" s="30" t="inlineStr">
         <is>
-          <t>Dracula terrorizes Transylvania and can found the Vampire Kingdom, which attacks its former controller and England before threatening the world. The one-battalion “Count Dracula” unit decides the kingdom's fate, and neighbors receive the “Fear of Dracula” national spirit until they confront it.</t>
+          <t>A shadowy society known as “Secret Society Influence” affects a government's ministers and generals, causing confusion and distrust. The national spirit reduces stability and political power while increasing consumer goods demand.</t>
         </is>
       </c>
       <c r="D141" s="35" t="n"/>
@@ -7581,22 +7585,26 @@
     </row>
     <row r="142" ht="22.5" customHeight="1">
       <c r="A142" s="34" t="n">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="B142" s="30" t="inlineStr">
         <is>
-          <t>Mass suicides</t>
+          <t>Teleportation Experiment</t>
         </is>
       </c>
       <c r="C142" s="30" t="inlineStr">
         <is>
-          <t>Whispers drive mass suicides in a random major country or the player. As deaths spread, generals and leaders can disappear until the country itself collapses.</t>
+          <t>A teleportation experiment makes one division vanish. A later breakthrough can move several divisions and shorten the cooldown.</t>
         </is>
       </c>
       <c r="D142" s="35" t="n"/>
       <c r="E142" s="36" t="n"/>
       <c r="F142" s="37" t="n"/>
-      <c r="G142" s="38" t="n"/>
+      <c r="G142" s="85" t="inlineStr">
+        <is>
+          <t>A teleportation breakthrough moves multiple divisions and shortens the cooldown.</t>
+        </is>
+      </c>
       <c r="H142" s="39" t="n"/>
       <c r="I142" s="40" t="n"/>
       <c r="J142" s="43" t="n"/>
@@ -7610,16 +7618,16 @@
     </row>
     <row r="143" ht="22.5" customHeight="1">
       <c r="A143" s="34" t="n">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="B143" s="30" t="inlineStr">
         <is>
-          <t>Partisans</t>
+          <t>Conspiracy Theorists</t>
         </is>
       </c>
       <c r="C143" s="30" t="inlineStr">
         <is>
-          <t>A major country or player with strong ideological support faces partisan divisions, some of them armored, in proportion to its support.</t>
+          <t>A conspiracy-theorist movement forms.</t>
         </is>
       </c>
       <c r="D143" s="35" t="n"/>
@@ -7639,16 +7647,16 @@
     </row>
     <row r="144" ht="22.5" customHeight="1">
       <c r="A144" s="34" t="n">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="B144" s="30" t="inlineStr">
         <is>
-          <t>A Game</t>
+          <t>Random Guarantee</t>
         </is>
       </c>
       <c r="C144" s="30" t="inlineStr">
         <is>
-          <t>A rock-paper-scissors contest decides a territorial dispute. Victory transfers the state, while defeat costs part of the player's industry.</t>
+          <t>A random major country guarantees a random minor.</t>
         </is>
       </c>
       <c r="D144" s="35" t="n"/>
@@ -7668,16 +7676,16 @@
     </row>
     <row r="145" ht="22.5" customHeight="1">
       <c r="A145" s="34" t="n">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="B145" s="30" t="inlineStr">
         <is>
-          <t>Freedom or Death</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="C145" s="30" t="inlineStr">
         <is>
-          <t>Subjects across the world declare independence and form the National Liberation Front. Their former masters can accept the separation or fight the simultaneous wars.</t>
+          <t>New Zealand begins questioning its own existence.</t>
         </is>
       </c>
       <c r="D145" s="35" t="n"/>
@@ -7697,16 +7705,16 @@
     </row>
     <row r="146" ht="22.5" customHeight="1">
       <c r="A146" s="34" t="n">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="B146" s="30" t="inlineStr">
         <is>
-          <t>The Book</t>
+          <t>Prophet</t>
         </is>
       </c>
       <c r="C146" s="30" t="inlineStr">
         <is>
-          <t>Intelligence agencies expand their clandestine networks.</t>
+          <t>A prophet travels the world preaching peace, leaving sayings in every country he visits.</t>
         </is>
       </c>
       <c r="D146" s="35" t="n"/>
@@ -7726,16 +7734,16 @@
     </row>
     <row r="147" ht="22.5" customHeight="1">
       <c r="A147" s="34" t="n">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="B147" s="30" t="inlineStr">
         <is>
-          <t>Add operative</t>
+          <t>Great Success</t>
         </is>
       </c>
       <c r="C147" s="30" t="inlineStr">
         <is>
-          <t>Counterintelligence improves across the world.</t>
+          <t>A travelling man reaches the United States and leaves behind a series of disruptive events.</t>
         </is>
       </c>
       <c r="D147" s="35" t="n"/>
@@ -7755,16 +7763,16 @@
     </row>
     <row r="148" ht="22.5" customHeight="1">
       <c r="A148" s="34" t="n">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="B148" s="30" t="inlineStr">
         <is>
-          <t>Counterintelligence</t>
+          <t>Change capital</t>
         </is>
       </c>
       <c r="C148" s="30" t="inlineStr">
         <is>
-          <t>Every country gains one point of counterintelligence.</t>
+          <t>Every country moves its capital to a random state.</t>
         </is>
       </c>
       <c r="D148" s="35" t="n"/>
@@ -7784,16 +7792,16 @@
     </row>
     <row r="149" ht="22.5" customHeight="1">
       <c r="A149" s="34" t="n">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="B149" s="30" t="inlineStr">
         <is>
-          <t>Pacifism</t>
+          <t>Tomorrow's Girls</t>
         </is>
       </c>
       <c r="C149" s="30" t="inlineStr">
         <is>
-          <t>Pacifism rises again as a political force.</t>
+          <t>An alien invasion begins through the mysterious song "Tomorrow's Girls" by Donald Fagen. A social game asks whether each girl is human or alien.</t>
         </is>
       </c>
       <c r="D149" s="35" t="n"/>
@@ -7813,16 +7821,16 @@
     </row>
     <row r="150" ht="22.5" customHeight="1">
       <c r="A150" s="34" t="n">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="B150" s="30" t="inlineStr">
         <is>
-          <t>Immigrations</t>
+          <t>The Free World</t>
         </is>
       </c>
       <c r="C150" s="30" t="inlineStr">
         <is>
-          <t>Retired and absorbed into the separate famine and migration mechanics through explicit adapters. Unavailable as a random event.</t>
+          <t>A vision of a unified world of salads and sun spreads across the campaign.</t>
         </is>
       </c>
       <c r="D150" s="35" t="n"/>
@@ -7842,16 +7850,16 @@
     </row>
     <row r="151" ht="22.5" customHeight="1">
       <c r="A151" s="34" t="n">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="B151" s="30" t="inlineStr">
         <is>
-          <t>Secret Society Influence</t>
+          <t>Shark infested waters</t>
         </is>
       </c>
       <c r="C151" s="30" t="inlineStr">
         <is>
-          <t>A shadowy society known as “Secret Society Influence” affects a government's ministers and generals, causing confusion and distrust. The national spirit reduces stability and political power while increasing consumer goods demand.</t>
+          <t>Shark-infested waters increase casualties whenever ships sink.</t>
         </is>
       </c>
       <c r="D151" s="35" t="n"/>
@@ -7871,16 +7879,16 @@
     </row>
     <row r="152" ht="22.5" customHeight="1">
       <c r="A152" s="34" t="n">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="B152" s="30" t="inlineStr">
         <is>
-          <t>Teleportation Experiment</t>
+          <t>Deal with the Devil</t>
         </is>
       </c>
       <c r="C152" s="30" t="inlineStr">
         <is>
-          <t>A teleportation experiment makes one division vanish. A later breakthrough can move several divisions and shorten the cooldown.</t>
+          <t>The Devil offers power in exchange for escalating bargains. Accepting more deals deepens the demonic influence, while refusal can bring new offers and harsher consequences before the pact is broken.</t>
         </is>
       </c>
       <c r="D152" s="35" t="n"/>
@@ -7888,7 +7896,7 @@
       <c r="F152" s="37" t="n"/>
       <c r="G152" s="85" t="inlineStr">
         <is>
-          <t>A teleportation breakthrough moves multiple divisions and shortens the cooldown.</t>
+          <t>The demonic influence reaches a second visual stage, with the leader's eyes changing.</t>
         </is>
       </c>
       <c r="H152" s="39" t="n"/>
@@ -7904,16 +7912,16 @@
     </row>
     <row r="153" ht="22.5" customHeight="1">
       <c r="A153" s="34" t="n">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="B153" s="30" t="inlineStr">
         <is>
-          <t>Conspiracy Theorists</t>
+          <t>Tin foil hat</t>
         </is>
       </c>
       <c r="C153" s="30" t="inlineStr">
         <is>
-          <t>A conspiracy-theorist movement forms.</t>
+          <t>Alien fears lead the United States to form an anti-alien coalition, with its leader adopting a tinfoil hat.</t>
         </is>
       </c>
       <c r="D153" s="35" t="n"/>
@@ -7933,16 +7941,16 @@
     </row>
     <row r="154" ht="22.5" customHeight="1">
       <c r="A154" s="34" t="n">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="B154" s="30" t="inlineStr">
         <is>
-          <t>Random Guarantee</t>
+          <t>Mr. LaPage</t>
         </is>
       </c>
       <c r="C154" s="30" t="inlineStr">
         <is>
-          <t>A random major country guarantees a random minor.</t>
+          <t>Mr. LaPage is a dangerous kidnapper inspired by the song Everyone's Gone to the Movies.</t>
         </is>
       </c>
       <c r="D154" s="35" t="n"/>
@@ -7962,16 +7970,16 @@
     </row>
     <row r="155" ht="22.5" customHeight="1">
       <c r="A155" s="34" t="n">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="B155" s="30" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Kamakiriad</t>
         </is>
       </c>
       <c r="C155" s="30" t="inlineStr">
         <is>
-          <t>New Zealand begins questioning its own existence.</t>
+          <t>A futuristic car travels the world.</t>
         </is>
       </c>
       <c r="D155" s="35" t="n"/>
@@ -7991,16 +7999,16 @@
     </row>
     <row r="156" ht="22.5" customHeight="1">
       <c r="A156" s="34" t="n">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="B156" s="30" t="inlineStr">
         <is>
-          <t>Prophet</t>
+          <t>The Custerdome</t>
         </is>
       </c>
       <c r="C156" s="30" t="inlineStr">
         <is>
-          <t>A prophet travels the world preaching peace, leaving sayings in every country he visits.</t>
+          <t>The campaign can end in the Custerdome when chaos stays low through 1944, opening a rare place of wealth and peace.</t>
         </is>
       </c>
       <c r="D156" s="35" t="n"/>
@@ -8009,7 +8017,11 @@
       <c r="G156" s="38" t="n"/>
       <c r="H156" s="39" t="n"/>
       <c r="I156" s="40" t="n"/>
-      <c r="J156" s="43" t="n"/>
+      <c r="J156" s="66" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
       <c r="K156" s="54" t="n"/>
       <c r="L156" s="54" t="n"/>
       <c r="M156" s="73" t="inlineStr">
@@ -8019,302 +8031,154 @@
       </c>
     </row>
     <row r="157" ht="22.5" customHeight="1">
-      <c r="A157" s="34" t="n">
-        <v>156</v>
-      </c>
-      <c r="B157" s="30" t="inlineStr">
-        <is>
-          <t>Great Success</t>
-        </is>
-      </c>
-      <c r="C157" s="30" t="inlineStr">
-        <is>
-          <t>A travelling man reaches the United States and leaves behind a series of disruptive events.</t>
-        </is>
-      </c>
-      <c r="D157" s="35" t="n"/>
-      <c r="E157" s="36" t="n"/>
-      <c r="F157" s="37" t="n"/>
-      <c r="G157" s="38" t="n"/>
-      <c r="H157" s="39" t="n"/>
-      <c r="I157" s="40" t="n"/>
-      <c r="J157" s="43" t="n"/>
-      <c r="K157" s="54" t="n"/>
-      <c r="L157" s="54" t="n"/>
-      <c r="M157" s="73" t="inlineStr">
-        <is>
-          <t>Unavailable</t>
-        </is>
-      </c>
+      <c r="A157" s="34"/>
+      <c r="B157" s="30"/>
+      <c r="C157" s="30"/>
+      <c r="D157" s="35"/>
+      <c r="E157" s="36"/>
+      <c r="F157" s="37"/>
+      <c r="G157" s="38"/>
+      <c r="H157" s="39"/>
+      <c r="I157" s="40"/>
+      <c r="J157" s="43"/>
+      <c r="K157" s="54"/>
+      <c r="L157" s="54"/>
+      <c r="M157" s="73"/>
     </row>
     <row r="158" ht="22.5" customHeight="1">
-      <c r="A158" s="34" t="n">
-        <v>157</v>
-      </c>
-      <c r="B158" s="30" t="inlineStr">
-        <is>
-          <t>Change capital</t>
-        </is>
-      </c>
-      <c r="C158" s="30" t="inlineStr">
-        <is>
-          <t>Every country moves its capital to a random state.</t>
-        </is>
-      </c>
-      <c r="D158" s="35" t="n"/>
-      <c r="E158" s="36" t="n"/>
-      <c r="F158" s="37" t="n"/>
-      <c r="G158" s="38" t="n"/>
-      <c r="H158" s="39" t="n"/>
-      <c r="I158" s="40" t="n"/>
-      <c r="J158" s="43" t="n"/>
-      <c r="K158" s="54" t="n"/>
-      <c r="L158" s="54" t="n"/>
-      <c r="M158" s="73" t="inlineStr">
-        <is>
-          <t>Unavailable</t>
-        </is>
-      </c>
+      <c r="A158" s="34"/>
+      <c r="B158" s="30"/>
+      <c r="C158" s="30"/>
+      <c r="D158" s="35"/>
+      <c r="E158" s="36"/>
+      <c r="F158" s="37"/>
+      <c r="G158" s="38"/>
+      <c r="H158" s="39"/>
+      <c r="I158" s="40"/>
+      <c r="J158" s="43"/>
+      <c r="K158" s="54"/>
+      <c r="L158" s="54"/>
+      <c r="M158" s="73"/>
     </row>
     <row r="159" ht="22.5" customHeight="1">
-      <c r="A159" s="34" t="n">
-        <v>158</v>
-      </c>
-      <c r="B159" s="30" t="inlineStr">
-        <is>
-          <t>Tomorrow's Girls</t>
-        </is>
-      </c>
-      <c r="C159" s="30" t="inlineStr">
-        <is>
-          <t>An alien invasion begins through the mysterious song "Tomorrow's Girls" by Donald Fagen. A social game asks whether each girl is human or alien.</t>
-        </is>
-      </c>
-      <c r="D159" s="35" t="n"/>
-      <c r="E159" s="36" t="n"/>
-      <c r="F159" s="37" t="n"/>
-      <c r="G159" s="38" t="n"/>
-      <c r="H159" s="39" t="n"/>
-      <c r="I159" s="40" t="n"/>
-      <c r="J159" s="43" t="n"/>
-      <c r="K159" s="54" t="n"/>
-      <c r="L159" s="54" t="n"/>
-      <c r="M159" s="73" t="inlineStr">
-        <is>
-          <t>Unavailable</t>
-        </is>
-      </c>
+      <c r="A159" s="34"/>
+      <c r="B159" s="30"/>
+      <c r="C159" s="30"/>
+      <c r="D159" s="35"/>
+      <c r="E159" s="36"/>
+      <c r="F159" s="37"/>
+      <c r="G159" s="38"/>
+      <c r="H159" s="39"/>
+      <c r="I159" s="40"/>
+      <c r="J159" s="43"/>
+      <c r="K159" s="54"/>
+      <c r="L159" s="54"/>
+      <c r="M159" s="73"/>
     </row>
     <row r="160" ht="22.5" customHeight="1">
-      <c r="A160" s="34" t="n">
-        <v>159</v>
-      </c>
-      <c r="B160" s="30" t="inlineStr">
-        <is>
-          <t>The Free World</t>
-        </is>
-      </c>
-      <c r="C160" s="30" t="inlineStr">
-        <is>
-          <t>A vision of a unified world of salads and sun spreads across the campaign.</t>
-        </is>
-      </c>
-      <c r="D160" s="35" t="n"/>
-      <c r="E160" s="36" t="n"/>
-      <c r="F160" s="37" t="n"/>
-      <c r="G160" s="38" t="n"/>
-      <c r="H160" s="39" t="n"/>
-      <c r="I160" s="40" t="n"/>
-      <c r="J160" s="43" t="n"/>
-      <c r="K160" s="54" t="n"/>
-      <c r="L160" s="54" t="n"/>
-      <c r="M160" s="73" t="inlineStr">
-        <is>
-          <t>Unavailable</t>
-        </is>
-      </c>
+      <c r="A160" s="34"/>
+      <c r="B160" s="30"/>
+      <c r="C160" s="30"/>
+      <c r="D160" s="35"/>
+      <c r="E160" s="36"/>
+      <c r="F160" s="37"/>
+      <c r="G160" s="38"/>
+      <c r="H160" s="39"/>
+      <c r="I160" s="40"/>
+      <c r="J160" s="43"/>
+      <c r="K160" s="54"/>
+      <c r="L160" s="54"/>
+      <c r="M160" s="73"/>
     </row>
     <row r="161" ht="22.5" customHeight="1">
-      <c r="A161" s="34" t="n">
-        <v>160</v>
-      </c>
-      <c r="B161" s="30" t="inlineStr">
-        <is>
-          <t>Shark infested waters</t>
-        </is>
-      </c>
-      <c r="C161" s="30" t="inlineStr">
-        <is>
-          <t>Shark-infested waters increase casualties whenever ships sink.</t>
-        </is>
-      </c>
-      <c r="D161" s="35" t="n"/>
-      <c r="E161" s="36" t="n"/>
-      <c r="F161" s="37" t="n"/>
-      <c r="G161" s="38" t="n"/>
-      <c r="H161" s="39" t="n"/>
-      <c r="I161" s="40" t="n"/>
-      <c r="J161" s="43" t="n"/>
-      <c r="K161" s="54" t="n"/>
-      <c r="L161" s="54" t="n"/>
-      <c r="M161" s="73" t="inlineStr">
-        <is>
-          <t>Unavailable</t>
-        </is>
-      </c>
+      <c r="A161" s="34"/>
+      <c r="B161" s="30"/>
+      <c r="C161" s="30"/>
+      <c r="D161" s="35"/>
+      <c r="E161" s="36"/>
+      <c r="F161" s="37"/>
+      <c r="G161" s="38"/>
+      <c r="H161" s="39"/>
+      <c r="I161" s="40"/>
+      <c r="J161" s="43"/>
+      <c r="K161" s="54"/>
+      <c r="L161" s="54"/>
+      <c r="M161" s="73"/>
     </row>
     <row r="162" ht="22.5" customHeight="1">
-      <c r="A162" s="34" t="n">
-        <v>161</v>
-      </c>
-      <c r="B162" s="30" t="inlineStr">
-        <is>
-          <t>Deal with the Devil</t>
-        </is>
-      </c>
-      <c r="C162" s="30" t="inlineStr">
-        <is>
-          <t>The Devil offers power in exchange for escalating bargains. Accepting more deals deepens the demonic influence, while refusal can bring new offers and harsher consequences before the pact is broken.</t>
-        </is>
-      </c>
-      <c r="D162" s="35" t="n"/>
-      <c r="E162" s="36" t="n"/>
-      <c r="F162" s="37" t="n"/>
-      <c r="G162" s="85" t="inlineStr">
-        <is>
-          <t>The demonic influence reaches a second visual stage, with the leader's eyes changing.</t>
-        </is>
-      </c>
-      <c r="H162" s="39" t="n"/>
-      <c r="I162" s="40" t="n"/>
-      <c r="J162" s="43" t="n"/>
-      <c r="K162" s="54" t="n"/>
-      <c r="L162" s="54" t="n"/>
-      <c r="M162" s="73" t="inlineStr">
-        <is>
-          <t>Unavailable</t>
-        </is>
-      </c>
+      <c r="A162" s="34"/>
+      <c r="B162" s="30"/>
+      <c r="C162" s="30"/>
+      <c r="D162" s="35"/>
+      <c r="E162" s="36"/>
+      <c r="F162" s="37"/>
+      <c r="G162" s="85"/>
+      <c r="H162" s="39"/>
+      <c r="I162" s="40"/>
+      <c r="J162" s="43"/>
+      <c r="K162" s="54"/>
+      <c r="L162" s="54"/>
+      <c r="M162" s="73"/>
     </row>
     <row r="163" ht="22.5" customHeight="1">
-      <c r="A163" s="34" t="n">
-        <v>162</v>
-      </c>
-      <c r="B163" s="30" t="inlineStr">
-        <is>
-          <t>Tin foil hat</t>
-        </is>
-      </c>
-      <c r="C163" s="30" t="inlineStr">
-        <is>
-          <t>Alien fears lead the United States to form an anti-alien coalition, with its leader adopting a tinfoil hat.</t>
-        </is>
-      </c>
-      <c r="D163" s="35" t="n"/>
-      <c r="E163" s="36" t="n"/>
-      <c r="F163" s="37" t="n"/>
-      <c r="G163" s="38" t="n"/>
-      <c r="H163" s="39" t="n"/>
-      <c r="I163" s="40" t="n"/>
-      <c r="J163" s="43" t="n"/>
-      <c r="K163" s="54" t="n"/>
-      <c r="L163" s="54" t="n"/>
-      <c r="M163" s="73" t="inlineStr">
-        <is>
-          <t>Unavailable</t>
-        </is>
-      </c>
+      <c r="A163" s="34"/>
+      <c r="B163" s="30"/>
+      <c r="C163" s="30"/>
+      <c r="D163" s="35"/>
+      <c r="E163" s="36"/>
+      <c r="F163" s="37"/>
+      <c r="G163" s="38"/>
+      <c r="H163" s="39"/>
+      <c r="I163" s="40"/>
+      <c r="J163" s="43"/>
+      <c r="K163" s="54"/>
+      <c r="L163" s="54"/>
+      <c r="M163" s="73"/>
     </row>
     <row r="164" ht="22.5" customHeight="1">
-      <c r="A164" s="34" t="n">
-        <v>164</v>
-      </c>
-      <c r="B164" s="30" t="inlineStr">
-        <is>
-          <t>Mr. LaPage</t>
-        </is>
-      </c>
-      <c r="C164" s="30" t="inlineStr">
-        <is>
-          <t>Mr. LaPage is a dangerous kidnapper inspired by the song Everyone's Gone to the Movies.</t>
-        </is>
-      </c>
-      <c r="D164" s="35" t="n"/>
-      <c r="E164" s="36" t="n"/>
-      <c r="F164" s="37" t="n"/>
-      <c r="G164" s="38" t="n"/>
-      <c r="H164" s="39" t="n"/>
-      <c r="I164" s="40" t="n"/>
-      <c r="J164" s="43" t="n"/>
-      <c r="K164" s="54" t="n"/>
-      <c r="L164" s="54" t="n"/>
-      <c r="M164" s="73" t="inlineStr">
-        <is>
-          <t>Unavailable</t>
-        </is>
-      </c>
+      <c r="A164" s="34"/>
+      <c r="B164" s="30"/>
+      <c r="C164" s="30"/>
+      <c r="D164" s="35"/>
+      <c r="E164" s="36"/>
+      <c r="F164" s="37"/>
+      <c r="G164" s="38"/>
+      <c r="H164" s="39"/>
+      <c r="I164" s="40"/>
+      <c r="J164" s="43"/>
+      <c r="K164" s="54"/>
+      <c r="L164" s="54"/>
+      <c r="M164" s="73"/>
     </row>
     <row r="165" ht="22.5" customHeight="1">
-      <c r="A165" s="34" t="n">
-        <v>165</v>
-      </c>
-      <c r="B165" s="30" t="inlineStr">
-        <is>
-          <t>Kamakiriad</t>
-        </is>
-      </c>
-      <c r="C165" s="30" t="inlineStr">
-        <is>
-          <t>A futuristic car travels the world.</t>
-        </is>
-      </c>
-      <c r="D165" s="35" t="n"/>
-      <c r="E165" s="36" t="n"/>
-      <c r="F165" s="37" t="n"/>
-      <c r="G165" s="38" t="n"/>
-      <c r="H165" s="39" t="n"/>
-      <c r="I165" s="40" t="n"/>
-      <c r="J165" s="43" t="n"/>
-      <c r="K165" s="54" t="n"/>
-      <c r="L165" s="54" t="n"/>
-      <c r="M165" s="73" t="inlineStr">
-        <is>
-          <t>Unavailable</t>
-        </is>
-      </c>
+      <c r="A165" s="34"/>
+      <c r="B165" s="30"/>
+      <c r="C165" s="30"/>
+      <c r="D165" s="35"/>
+      <c r="E165" s="36"/>
+      <c r="F165" s="37"/>
+      <c r="G165" s="38"/>
+      <c r="H165" s="39"/>
+      <c r="I165" s="40"/>
+      <c r="J165" s="43"/>
+      <c r="K165" s="54"/>
+      <c r="L165" s="54"/>
+      <c r="M165" s="73"/>
     </row>
     <row r="166" ht="22.5" customHeight="1">
-      <c r="A166" s="34" t="n">
-        <v>166</v>
-      </c>
-      <c r="B166" s="30" t="inlineStr">
-        <is>
-          <t>The Custerdome</t>
-        </is>
-      </c>
-      <c r="C166" s="30" t="inlineStr">
-        <is>
-          <t>The campaign can end in the Custerdome when chaos stays low through 1944, opening a rare place of wealth and peace.</t>
-        </is>
-      </c>
-      <c r="D166" s="35" t="n"/>
-      <c r="E166" s="36" t="n"/>
-      <c r="F166" s="37" t="n"/>
-      <c r="G166" s="38" t="n"/>
-      <c r="H166" s="39" t="n"/>
-      <c r="I166" s="40" t="n"/>
-      <c r="J166" s="66" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="K166" s="54" t="n"/>
-      <c r="L166" s="54" t="n"/>
-      <c r="M166" s="73" t="inlineStr">
-        <is>
-          <t>Unavailable</t>
-        </is>
-      </c>
+      <c r="A166" s="34"/>
+      <c r="B166" s="30"/>
+      <c r="C166" s="30"/>
+      <c r="D166" s="35"/>
+      <c r="E166" s="36"/>
+      <c r="F166" s="37"/>
+      <c r="G166" s="38"/>
+      <c r="H166" s="39"/>
+      <c r="I166" s="40"/>
+      <c r="J166" s="66"/>
+      <c r="K166" s="54"/>
+      <c r="L166" s="54"/>
+      <c r="M166" s="73"/>
     </row>
     <row r="167" ht="22.5" customHeight="1">
       <c r="A167" s="34" t="n"/>
@@ -21557,12 +21421,12 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>42, 47</t>
+          <t>42, 47, 109</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Low, Low</t>
+          <t>Low, Low, Severe</t>
         </is>
       </c>
       <c r="F12" s="68" t="inlineStr">
@@ -21953,7 +21817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -24113,6 +23977,37 @@
       <c r="G77" s="5" t="inlineStr">
         <is>
           <t>Also Sudden Abundance at Medium severity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Various Anomalies</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D78" s="5" t="n">
+        <v>109</v>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>Fuel Crisis</t>
+        </is>
+      </c>
+      <c r="F78" s="54" t="inlineStr">
+        <is>
+          <t>Severe</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>Worldwide fuel reserve loss. Canonical event identity 109, former catalog identity 114.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align Event 033 catalog text and update the 028 and 033 validators
The Event 033 and Natural Disasters catalog descriptions now match the
restored in-game localisation, and the CSV exports are regenerated.

The Event 028 availability validator accepts the reopened board's refresh
block and compares the complete option pools of the paginated boards.
The Event 033 validator checks the restored cluster pacing contract
instead of the removed mixed-Major override.

The tooling plan records step 1 and the owner hand-offs.
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -3849,7 +3849,7 @@
       </c>
       <c r="C34" s="30" t="inlineStr">
         <is>
-          <t>A lethal acid-rain system moves between regions, exposing the inhabited states in its path to corrosion, poisoned runoff, infrastructure damage, and direct civilian loss. Countries can build shelters, protect water and food, expand emergency medicine, harden transport, evacuate states ahead of storm forecasts, and repair the aftermath. The rain ordinarily disperses only after it has crossed every state in its path.</t>
+          <t>A lethal acid-rain system moves between regions, exposing the inhabited states registered at formation to corrosion, poisoned runoff, infrastructure damage, and direct civilian loss. Countries can build shelters, protect water and food, expand emergency medicine, harden transport, evacuate states ahead of storm forecasts, and repair the aftermath. The rain ordinarily disperses only after it has crossed every eligible state.</t>
         </is>
       </c>
       <c r="D34" s="35" t="inlineStr">
@@ -21188,7 +21188,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Natural and environmental catastrophes strike states or regions, with repeated disaster slots allowing the cluster to scale into larger cascades.</t>
+          <t>Natural Disasters can strike repeatedly across distant states. Early crises remain local, while higher chaos brings regional cascades and disasters that move along abnormal paths. Each affected country receives its own reports and recovery work.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Import event planning packages 123, 124, 131 and 132
Install the Equipment choice, Sun moves away, Immigrations and Secret Society
Influence packages under docs/specs with their historical evidence and import
handoffs under docs/plans, reconciled with current repository guidance.

Adopt the package identities in the event catalog and shared identifier
registry (former catalog IDs 135, 136, 149 and 150), and record Event 131 as
the superseding identity of retired Event 149 in the migration documents.
No gameplay files changed and nothing was run in engine.
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -7063,16 +7063,16 @@
     </row>
     <row r="124" ht="22.5" customHeight="1">
       <c r="A124" s="34" t="n">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B124" s="30" t="inlineStr">
         <is>
-          <t>Non-Aggressions</t>
+          <t>Equipment choice</t>
         </is>
       </c>
       <c r="C124" s="30" t="inlineStr">
         <is>
-          <t>Two random countries sign a non-aggression pact.</t>
+          <t>Every country receives a choice of large equipment grants.</t>
         </is>
       </c>
       <c r="D124" s="35" t="n"/>
@@ -7092,16 +7092,16 @@
     </row>
     <row r="125" ht="22.5" customHeight="1">
       <c r="A125" s="34" t="n">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B125" s="30" t="inlineStr">
         <is>
-          <t>Duchies</t>
+          <t>Sun moves away</t>
         </is>
       </c>
       <c r="C125" s="30" t="inlineStr">
         <is>
-          <t>Countries face a sudden surplus of military equipment.</t>
+          <t>The Sun moves away, leaving the whole world in continuous darkness and unnatural winter until it returns.</t>
         </is>
       </c>
       <c r="D125" s="35" t="n"/>
@@ -7121,16 +7121,16 @@
     </row>
     <row r="126" ht="22.5" customHeight="1">
       <c r="A126" s="34" t="n">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="B126" s="30" t="inlineStr">
         <is>
-          <t>Equipment choice</t>
+          <t>Non-Aggressions</t>
         </is>
       </c>
       <c r="C126" s="30" t="inlineStr">
         <is>
-          <t>Every country receives a choice of large equipment grants.</t>
+          <t>Two random countries sign a non-aggression pact.</t>
         </is>
       </c>
       <c r="D126" s="35" t="n"/>
@@ -7150,16 +7150,16 @@
     </row>
     <row r="127" ht="22.5" customHeight="1">
       <c r="A127" s="34" t="n">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B127" s="30" t="inlineStr">
         <is>
-          <t>Sun moves away</t>
+          <t>Immigrations</t>
         </is>
       </c>
       <c r="C127" s="30" t="inlineStr">
         <is>
-          <t>A research surge focuses each country on one field.</t>
+          <t>Waves of people leave their homes for a foreign country, and governments choose how to receive them.</t>
         </is>
       </c>
       <c r="D127" s="35" t="n"/>
@@ -7179,16 +7179,16 @@
     </row>
     <row r="128" ht="22.5" customHeight="1">
       <c r="A128" s="34" t="n">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B128" s="30" t="inlineStr">
         <is>
-          <t>Research Investment</t>
+          <t>Secret Society Influence</t>
         </is>
       </c>
       <c r="C128" s="30" t="inlineStr">
         <is>
-          <t>Every country receives a choice of research investment in one category.</t>
+          <t>A shadowy society known as “Secret Society Influence” affects a government's ministers and generals, causing confusion and distrust. The national spirit reduces stability and political power while increasing consumer goods demand.</t>
         </is>
       </c>
       <c r="D128" s="35" t="n"/>
@@ -7208,16 +7208,16 @@
     </row>
     <row r="129" ht="22.5" customHeight="1">
       <c r="A129" s="34" t="n">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B129" s="30" t="inlineStr">
         <is>
-          <t>The Kingdom of the Mountains</t>
+          <t>Duchies</t>
         </is>
       </c>
       <c r="C129" s="30" t="inlineStr">
         <is>
-          <t>A mountain and hill country forms the Mountain Republic and claims every matching state.</t>
+          <t>Countries face a sudden surplus of military equipment.</t>
         </is>
       </c>
       <c r="D129" s="35" t="n"/>
@@ -7237,16 +7237,16 @@
     </row>
     <row r="130" ht="22.5" customHeight="1">
       <c r="A130" s="34" t="n">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B130" s="30" t="inlineStr">
         <is>
-          <t>Mysterious creature</t>
+          <t>Research Investment</t>
         </is>
       </c>
       <c r="C130" s="30" t="inlineStr">
         <is>
-          <t>A creature feeds on crops and people in a random major country or the player, spreading fear until it is hunted.</t>
+          <t>Every country receives a choice of research investment in one category.</t>
         </is>
       </c>
       <c r="D130" s="35" t="n"/>
@@ -7266,16 +7266,16 @@
     </row>
     <row r="131" ht="22.5" customHeight="1">
       <c r="A131" s="34" t="n">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B131" s="30" t="inlineStr">
         <is>
-          <t>Dracula</t>
+          <t>The Kingdom of the Mountains</t>
         </is>
       </c>
       <c r="C131" s="30" t="inlineStr">
         <is>
-          <t>Dracula terrorizes Transylvania and can found the Vampire Kingdom, which attacks its former controller and England before threatening the world. The one-battalion “Count Dracula” unit decides the kingdom's fate, and neighbors receive the “Fear of Dracula” national spirit until they confront it.</t>
+          <t>A mountain and hill country forms the Mountain Republic and claims every matching state.</t>
         </is>
       </c>
       <c r="D131" s="35" t="n"/>
@@ -7295,16 +7295,16 @@
     </row>
     <row r="132" ht="22.5" customHeight="1">
       <c r="A132" s="34" t="n">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B132" s="30" t="inlineStr">
         <is>
-          <t>Mass suicides</t>
+          <t>Mysterious creature</t>
         </is>
       </c>
       <c r="C132" s="30" t="inlineStr">
         <is>
-          <t>Whispers drive mass suicides in a random major country or the player. As deaths spread, generals and leaders can disappear until the country itself collapses.</t>
+          <t>A creature feeds on crops and people in a random major country or the player, spreading fear until it is hunted.</t>
         </is>
       </c>
       <c r="D132" s="35" t="n"/>
@@ -7324,16 +7324,16 @@
     </row>
     <row r="133" ht="22.5" customHeight="1">
       <c r="A133" s="34" t="n">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B133" s="30" t="inlineStr">
         <is>
-          <t>Partisans</t>
+          <t>Dracula</t>
         </is>
       </c>
       <c r="C133" s="30" t="inlineStr">
         <is>
-          <t>A major country or player with strong ideological support faces partisan divisions, some of them armored, in proportion to its support.</t>
+          <t>Dracula terrorizes Transylvania and can found the Vampire Kingdom, which attacks its former controller and England before threatening the world. The one-battalion “Count Dracula” unit decides the kingdom's fate, and neighbors receive the “Fear of Dracula” national spirit until they confront it.</t>
         </is>
       </c>
       <c r="D133" s="35" t="n"/>
@@ -7353,16 +7353,16 @@
     </row>
     <row r="134" ht="22.5" customHeight="1">
       <c r="A134" s="34" t="n">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B134" s="30" t="inlineStr">
         <is>
-          <t>A Game</t>
+          <t>Mass suicides</t>
         </is>
       </c>
       <c r="C134" s="30" t="inlineStr">
         <is>
-          <t>A rock-paper-scissors contest decides a territorial dispute. Victory transfers the state, while defeat costs part of the player's industry.</t>
+          <t>Whispers drive mass suicides in a random major country or the player. As deaths spread, generals and leaders can disappear until the country itself collapses.</t>
         </is>
       </c>
       <c r="D134" s="35" t="n"/>
@@ -7382,16 +7382,16 @@
     </row>
     <row r="135" ht="22.5" customHeight="1">
       <c r="A135" s="34" t="n">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B135" s="30" t="inlineStr">
         <is>
-          <t>Freedom or Death</t>
+          <t>Partisans</t>
         </is>
       </c>
       <c r="C135" s="30" t="inlineStr">
         <is>
-          <t>Subjects across the world declare independence and form the National Liberation Front. Their former masters can accept the separation or fight the simultaneous wars.</t>
+          <t>A major country or player with strong ideological support faces partisan divisions, some of them armored, in proportion to its support.</t>
         </is>
       </c>
       <c r="D135" s="35" t="n"/>
@@ -7411,16 +7411,16 @@
     </row>
     <row r="136" ht="22.5" customHeight="1">
       <c r="A136" s="34" t="n">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B136" s="30" t="inlineStr">
         <is>
-          <t>The Book</t>
+          <t>A Game</t>
         </is>
       </c>
       <c r="C136" s="30" t="inlineStr">
         <is>
-          <t>Intelligence agencies expand their clandestine networks.</t>
+          <t>A rock-paper-scissors contest decides a territorial dispute. Victory transfers the state, while defeat costs part of the player's industry.</t>
         </is>
       </c>
       <c r="D136" s="35" t="n"/>
@@ -7440,16 +7440,16 @@
     </row>
     <row r="137" ht="22.5" customHeight="1">
       <c r="A137" s="34" t="n">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B137" s="30" t="inlineStr">
         <is>
-          <t>Add operative</t>
+          <t>Freedom or Death</t>
         </is>
       </c>
       <c r="C137" s="30" t="inlineStr">
         <is>
-          <t>Counterintelligence improves across the world.</t>
+          <t>Subjects across the world declare independence and form the National Liberation Front. Their former masters can accept the separation or fight the simultaneous wars.</t>
         </is>
       </c>
       <c r="D137" s="35" t="n"/>
@@ -7469,16 +7469,16 @@
     </row>
     <row r="138" ht="22.5" customHeight="1">
       <c r="A138" s="34" t="n">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B138" s="30" t="inlineStr">
         <is>
-          <t>Counterintelligence</t>
+          <t>The Book</t>
         </is>
       </c>
       <c r="C138" s="30" t="inlineStr">
         <is>
-          <t>Every country gains one point of counterintelligence.</t>
+          <t>Intelligence agencies expand their clandestine networks.</t>
         </is>
       </c>
       <c r="D138" s="35" t="n"/>
@@ -7498,16 +7498,16 @@
     </row>
     <row r="139" ht="22.5" customHeight="1">
       <c r="A139" s="34" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B139" s="30" t="inlineStr">
         <is>
-          <t>Pacifism</t>
+          <t>Add operative</t>
         </is>
       </c>
       <c r="C139" s="30" t="inlineStr">
         <is>
-          <t>Pacifism rises again as a political force.</t>
+          <t>Counterintelligence improves across the world.</t>
         </is>
       </c>
       <c r="D139" s="35" t="n"/>
@@ -7527,16 +7527,16 @@
     </row>
     <row r="140" ht="22.5" customHeight="1">
       <c r="A140" s="34" t="n">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B140" s="30" t="inlineStr">
         <is>
-          <t>Immigrations</t>
+          <t>Counterintelligence</t>
         </is>
       </c>
       <c r="C140" s="30" t="inlineStr">
         <is>
-          <t>Retired and absorbed into the separate famine and migration mechanics through explicit adapters. Unavailable as a random event.</t>
+          <t>Every country gains one point of counterintelligence.</t>
         </is>
       </c>
       <c r="D140" s="35" t="n"/>
@@ -7556,16 +7556,16 @@
     </row>
     <row r="141" ht="22.5" customHeight="1">
       <c r="A141" s="34" t="n">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B141" s="30" t="inlineStr">
         <is>
-          <t>Secret Society Influence</t>
+          <t>Pacifism</t>
         </is>
       </c>
       <c r="C141" s="30" t="inlineStr">
         <is>
-          <t>A shadowy society known as “Secret Society Influence” affects a government's ministers and generals, causing confusion and distrust. The national spirit reduces stability and political power while increasing consumer goods demand.</t>
+          <t>Pacifism rises again as a political force.</t>
         </is>
       </c>
       <c r="D141" s="35" t="n"/>
@@ -8031,154 +8031,154 @@
       </c>
     </row>
     <row r="157" ht="22.5" customHeight="1">
-      <c r="A157" s="34"/>
-      <c r="B157" s="30"/>
-      <c r="C157" s="30"/>
-      <c r="D157" s="35"/>
-      <c r="E157" s="36"/>
-      <c r="F157" s="37"/>
-      <c r="G157" s="38"/>
-      <c r="H157" s="39"/>
-      <c r="I157" s="40"/>
-      <c r="J157" s="43"/>
-      <c r="K157" s="54"/>
-      <c r="L157" s="54"/>
-      <c r="M157" s="73"/>
+      <c r="A157" s="34" t="n"/>
+      <c r="B157" s="30" t="n"/>
+      <c r="C157" s="30" t="n"/>
+      <c r="D157" s="35" t="n"/>
+      <c r="E157" s="36" t="n"/>
+      <c r="F157" s="37" t="n"/>
+      <c r="G157" s="38" t="n"/>
+      <c r="H157" s="39" t="n"/>
+      <c r="I157" s="40" t="n"/>
+      <c r="J157" s="43" t="n"/>
+      <c r="K157" s="54" t="n"/>
+      <c r="L157" s="54" t="n"/>
+      <c r="M157" s="73" t="n"/>
     </row>
     <row r="158" ht="22.5" customHeight="1">
-      <c r="A158" s="34"/>
-      <c r="B158" s="30"/>
-      <c r="C158" s="30"/>
-      <c r="D158" s="35"/>
-      <c r="E158" s="36"/>
-      <c r="F158" s="37"/>
-      <c r="G158" s="38"/>
-      <c r="H158" s="39"/>
-      <c r="I158" s="40"/>
-      <c r="J158" s="43"/>
-      <c r="K158" s="54"/>
-      <c r="L158" s="54"/>
-      <c r="M158" s="73"/>
+      <c r="A158" s="34" t="n"/>
+      <c r="B158" s="30" t="n"/>
+      <c r="C158" s="30" t="n"/>
+      <c r="D158" s="35" t="n"/>
+      <c r="E158" s="36" t="n"/>
+      <c r="F158" s="37" t="n"/>
+      <c r="G158" s="38" t="n"/>
+      <c r="H158" s="39" t="n"/>
+      <c r="I158" s="40" t="n"/>
+      <c r="J158" s="43" t="n"/>
+      <c r="K158" s="54" t="n"/>
+      <c r="L158" s="54" t="n"/>
+      <c r="M158" s="73" t="n"/>
     </row>
     <row r="159" ht="22.5" customHeight="1">
-      <c r="A159" s="34"/>
-      <c r="B159" s="30"/>
-      <c r="C159" s="30"/>
-      <c r="D159" s="35"/>
-      <c r="E159" s="36"/>
-      <c r="F159" s="37"/>
-      <c r="G159" s="38"/>
-      <c r="H159" s="39"/>
-      <c r="I159" s="40"/>
-      <c r="J159" s="43"/>
-      <c r="K159" s="54"/>
-      <c r="L159" s="54"/>
-      <c r="M159" s="73"/>
+      <c r="A159" s="34" t="n"/>
+      <c r="B159" s="30" t="n"/>
+      <c r="C159" s="30" t="n"/>
+      <c r="D159" s="35" t="n"/>
+      <c r="E159" s="36" t="n"/>
+      <c r="F159" s="37" t="n"/>
+      <c r="G159" s="38" t="n"/>
+      <c r="H159" s="39" t="n"/>
+      <c r="I159" s="40" t="n"/>
+      <c r="J159" s="43" t="n"/>
+      <c r="K159" s="54" t="n"/>
+      <c r="L159" s="54" t="n"/>
+      <c r="M159" s="73" t="n"/>
     </row>
     <row r="160" ht="22.5" customHeight="1">
-      <c r="A160" s="34"/>
-      <c r="B160" s="30"/>
-      <c r="C160" s="30"/>
-      <c r="D160" s="35"/>
-      <c r="E160" s="36"/>
-      <c r="F160" s="37"/>
-      <c r="G160" s="38"/>
-      <c r="H160" s="39"/>
-      <c r="I160" s="40"/>
-      <c r="J160" s="43"/>
-      <c r="K160" s="54"/>
-      <c r="L160" s="54"/>
-      <c r="M160" s="73"/>
+      <c r="A160" s="34" t="n"/>
+      <c r="B160" s="30" t="n"/>
+      <c r="C160" s="30" t="n"/>
+      <c r="D160" s="35" t="n"/>
+      <c r="E160" s="36" t="n"/>
+      <c r="F160" s="37" t="n"/>
+      <c r="G160" s="38" t="n"/>
+      <c r="H160" s="39" t="n"/>
+      <c r="I160" s="40" t="n"/>
+      <c r="J160" s="43" t="n"/>
+      <c r="K160" s="54" t="n"/>
+      <c r="L160" s="54" t="n"/>
+      <c r="M160" s="73" t="n"/>
     </row>
     <row r="161" ht="22.5" customHeight="1">
-      <c r="A161" s="34"/>
-      <c r="B161" s="30"/>
-      <c r="C161" s="30"/>
-      <c r="D161" s="35"/>
-      <c r="E161" s="36"/>
-      <c r="F161" s="37"/>
-      <c r="G161" s="38"/>
-      <c r="H161" s="39"/>
-      <c r="I161" s="40"/>
-      <c r="J161" s="43"/>
-      <c r="K161" s="54"/>
-      <c r="L161" s="54"/>
-      <c r="M161" s="73"/>
+      <c r="A161" s="34" t="n"/>
+      <c r="B161" s="30" t="n"/>
+      <c r="C161" s="30" t="n"/>
+      <c r="D161" s="35" t="n"/>
+      <c r="E161" s="36" t="n"/>
+      <c r="F161" s="37" t="n"/>
+      <c r="G161" s="38" t="n"/>
+      <c r="H161" s="39" t="n"/>
+      <c r="I161" s="40" t="n"/>
+      <c r="J161" s="43" t="n"/>
+      <c r="K161" s="54" t="n"/>
+      <c r="L161" s="54" t="n"/>
+      <c r="M161" s="73" t="n"/>
     </row>
     <row r="162" ht="22.5" customHeight="1">
-      <c r="A162" s="34"/>
-      <c r="B162" s="30"/>
-      <c r="C162" s="30"/>
-      <c r="D162" s="35"/>
-      <c r="E162" s="36"/>
-      <c r="F162" s="37"/>
-      <c r="G162" s="85"/>
-      <c r="H162" s="39"/>
-      <c r="I162" s="40"/>
-      <c r="J162" s="43"/>
-      <c r="K162" s="54"/>
-      <c r="L162" s="54"/>
-      <c r="M162" s="73"/>
+      <c r="A162" s="34" t="n"/>
+      <c r="B162" s="30" t="n"/>
+      <c r="C162" s="30" t="n"/>
+      <c r="D162" s="35" t="n"/>
+      <c r="E162" s="36" t="n"/>
+      <c r="F162" s="37" t="n"/>
+      <c r="G162" s="85" t="n"/>
+      <c r="H162" s="39" t="n"/>
+      <c r="I162" s="40" t="n"/>
+      <c r="J162" s="43" t="n"/>
+      <c r="K162" s="54" t="n"/>
+      <c r="L162" s="54" t="n"/>
+      <c r="M162" s="73" t="n"/>
     </row>
     <row r="163" ht="22.5" customHeight="1">
-      <c r="A163" s="34"/>
-      <c r="B163" s="30"/>
-      <c r="C163" s="30"/>
-      <c r="D163" s="35"/>
-      <c r="E163" s="36"/>
-      <c r="F163" s="37"/>
-      <c r="G163" s="38"/>
-      <c r="H163" s="39"/>
-      <c r="I163" s="40"/>
-      <c r="J163" s="43"/>
-      <c r="K163" s="54"/>
-      <c r="L163" s="54"/>
-      <c r="M163" s="73"/>
+      <c r="A163" s="34" t="n"/>
+      <c r="B163" s="30" t="n"/>
+      <c r="C163" s="30" t="n"/>
+      <c r="D163" s="35" t="n"/>
+      <c r="E163" s="36" t="n"/>
+      <c r="F163" s="37" t="n"/>
+      <c r="G163" s="38" t="n"/>
+      <c r="H163" s="39" t="n"/>
+      <c r="I163" s="40" t="n"/>
+      <c r="J163" s="43" t="n"/>
+      <c r="K163" s="54" t="n"/>
+      <c r="L163" s="54" t="n"/>
+      <c r="M163" s="73" t="n"/>
     </row>
     <row r="164" ht="22.5" customHeight="1">
-      <c r="A164" s="34"/>
-      <c r="B164" s="30"/>
-      <c r="C164" s="30"/>
-      <c r="D164" s="35"/>
-      <c r="E164" s="36"/>
-      <c r="F164" s="37"/>
-      <c r="G164" s="38"/>
-      <c r="H164" s="39"/>
-      <c r="I164" s="40"/>
-      <c r="J164" s="43"/>
-      <c r="K164" s="54"/>
-      <c r="L164" s="54"/>
-      <c r="M164" s="73"/>
+      <c r="A164" s="34" t="n"/>
+      <c r="B164" s="30" t="n"/>
+      <c r="C164" s="30" t="n"/>
+      <c r="D164" s="35" t="n"/>
+      <c r="E164" s="36" t="n"/>
+      <c r="F164" s="37" t="n"/>
+      <c r="G164" s="38" t="n"/>
+      <c r="H164" s="39" t="n"/>
+      <c r="I164" s="40" t="n"/>
+      <c r="J164" s="43" t="n"/>
+      <c r="K164" s="54" t="n"/>
+      <c r="L164" s="54" t="n"/>
+      <c r="M164" s="73" t="n"/>
     </row>
     <row r="165" ht="22.5" customHeight="1">
-      <c r="A165" s="34"/>
-      <c r="B165" s="30"/>
-      <c r="C165" s="30"/>
-      <c r="D165" s="35"/>
-      <c r="E165" s="36"/>
-      <c r="F165" s="37"/>
-      <c r="G165" s="38"/>
-      <c r="H165" s="39"/>
-      <c r="I165" s="40"/>
-      <c r="J165" s="43"/>
-      <c r="K165" s="54"/>
-      <c r="L165" s="54"/>
-      <c r="M165" s="73"/>
+      <c r="A165" s="34" t="n"/>
+      <c r="B165" s="30" t="n"/>
+      <c r="C165" s="30" t="n"/>
+      <c r="D165" s="35" t="n"/>
+      <c r="E165" s="36" t="n"/>
+      <c r="F165" s="37" t="n"/>
+      <c r="G165" s="38" t="n"/>
+      <c r="H165" s="39" t="n"/>
+      <c r="I165" s="40" t="n"/>
+      <c r="J165" s="43" t="n"/>
+      <c r="K165" s="54" t="n"/>
+      <c r="L165" s="54" t="n"/>
+      <c r="M165" s="73" t="n"/>
     </row>
     <row r="166" ht="22.5" customHeight="1">
-      <c r="A166" s="34"/>
-      <c r="B166" s="30"/>
-      <c r="C166" s="30"/>
-      <c r="D166" s="35"/>
-      <c r="E166" s="36"/>
-      <c r="F166" s="37"/>
-      <c r="G166" s="38"/>
-      <c r="H166" s="39"/>
-      <c r="I166" s="40"/>
-      <c r="J166" s="66"/>
-      <c r="K166" s="54"/>
-      <c r="L166" s="54"/>
-      <c r="M166" s="73"/>
+      <c r="A166" s="34" t="n"/>
+      <c r="B166" s="30" t="n"/>
+      <c r="C166" s="30" t="n"/>
+      <c r="D166" s="35" t="n"/>
+      <c r="E166" s="36" t="n"/>
+      <c r="F166" s="37" t="n"/>
+      <c r="G166" s="38" t="n"/>
+      <c r="H166" s="39" t="n"/>
+      <c r="I166" s="40" t="n"/>
+      <c r="J166" s="66" t="n"/>
+      <c r="K166" s="54" t="n"/>
+      <c r="L166" s="54" t="n"/>
+      <c r="M166" s="73" t="n"/>
     </row>
     <row r="167" ht="22.5" customHeight="1">
       <c r="A167" s="34" t="n"/>

</xml_diff>